<commit_message>
added Manual test counts
</commit_message>
<xml_diff>
--- a/tests/Manual.Integration.Tests.xlsx
+++ b/tests/Manual.Integration.Tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Microsoft\ActiveDirectoryTierModel\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6A05EBA-E70C-40A0-80E3-BAB7BBE0DB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5017D7E2-C2B4-4D9B-B4A7-925418F8CE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="555" yWindow="45" windowWidth="37080" windowHeight="20880" xr2:uid="{C99BB6DE-AC80-4F97-BF9F-2DFD37C8A9E7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3952" uniqueCount="876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4242" uniqueCount="995">
   <si>
     <t>Test Num</t>
   </si>
@@ -2575,9 +2575,6 @@
 Domain Join an End-User Device to the Domain using a Tier 2 Account Service Account</t>
   </si>
   <si>
-    <t>Auth Silo - Allow Tier 0 PAW</t>
-  </si>
-  <si>
     <t>Auth Silo - Allow Tier 0 Member Server - Interactive</t>
   </si>
   <si>
@@ -2638,9 +2635,6 @@
     <t>Deploy Running FullDeployment &amp; Manage Service Accounts &amp; Windows LAPS &amp; Enable Auditing &amp; Auth Silos</t>
   </si>
   <si>
-    <t>Auth Silo - Allow Tier 1 PAW</t>
-  </si>
-  <si>
     <t>Auth Silo - Allow Tier 1 Member Server - Interactive</t>
   </si>
   <si>
@@ -2665,43 +2659,416 @@
     <t>Auth Silo - Reduced TGT Time</t>
   </si>
   <si>
-    <t>Klist shows 4 hour TGT with Tier 1 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Klist shows 2 hour TGT with Tier 0 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Auth Silo - Allow Tier 2 PAW</t>
-  </si>
-  <si>
-    <t>Klist shows 6 hour TGT with Tier 0 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
     <t>Auth Silo - Allow Tier 2 End-User Device - Interactive</t>
   </si>
   <si>
-    <t>Denied login with Tier 2 EUD Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Allowed to login with Tier 2 EUD Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Denied to login with Tier 0 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Allowed to login with Tier 2 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Allowed to login with Tier 1 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Denied login with Tier 1 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Allowed to login with Tier 0 Auth Silo Policy Enforced</t>
-  </si>
-  <si>
-    <t>Denied lgin with Tier 0 Auth Silo Policy Enforced</t>
+    <t>D-10</t>
+  </si>
+  <si>
+    <t>D-11</t>
+  </si>
+  <si>
+    <t>D-12</t>
+  </si>
+  <si>
+    <t>D-13</t>
+  </si>
+  <si>
+    <t>D-14</t>
+  </si>
+  <si>
+    <t>D-15</t>
+  </si>
+  <si>
+    <t>D-16</t>
+  </si>
+  <si>
+    <t>D-17</t>
+  </si>
+  <si>
+    <t>D-18</t>
+  </si>
+  <si>
+    <t>D-19</t>
+  </si>
+  <si>
+    <t>D-20</t>
+  </si>
+  <si>
+    <t>D-21</t>
+  </si>
+  <si>
+    <t>D-22</t>
+  </si>
+  <si>
+    <t>D-23</t>
+  </si>
+  <si>
+    <t>D-24</t>
+  </si>
+  <si>
+    <t>D-25</t>
+  </si>
+  <si>
+    <t>D-26</t>
+  </si>
+  <si>
+    <t>D-27</t>
+  </si>
+  <si>
+    <t>D-28</t>
+  </si>
+  <si>
+    <t>D-29</t>
+  </si>
+  <si>
+    <t>D-30</t>
+  </si>
+  <si>
+    <t>D-31</t>
+  </si>
+  <si>
+    <t>D-32</t>
+  </si>
+  <si>
+    <t>D-33</t>
+  </si>
+  <si>
+    <t>D-34</t>
+  </si>
+  <si>
+    <t>D-35</t>
+  </si>
+  <si>
+    <t>D-36</t>
+  </si>
+  <si>
+    <t>D-37</t>
+  </si>
+  <si>
+    <t>D-38</t>
+  </si>
+  <si>
+    <t>D-39</t>
+  </si>
+  <si>
+    <t>D-40</t>
+  </si>
+  <si>
+    <t>D-41</t>
+  </si>
+  <si>
+    <t>Auth Silo - Allow Tier 0 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>Auth Silo - Allow Tier 1 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>Auth Silo - Allow Tier 2 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>Tier 0 Operators
+Tier 0 Authentication Policy</t>
+  </si>
+  <si>
+    <t>Klist shows 2 hour TGT with Tier 0 Authentication Silo Policy Enforced</t>
+  </si>
+  <si>
+    <t>Tier 2 Operators
+Tier 2 Authentication Policy</t>
+  </si>
+  <si>
+    <t>Tier 2 Local Device Operators
+Tier 2 Authentication Policy</t>
+  </si>
+  <si>
+    <t>T2-062</t>
+  </si>
+  <si>
+    <t>T2-063</t>
+  </si>
+  <si>
+    <t>T2-064</t>
+  </si>
+  <si>
+    <t>T2-065</t>
+  </si>
+  <si>
+    <t>T2-066</t>
+  </si>
+  <si>
+    <t>T2-067</t>
+  </si>
+  <si>
+    <t>T2-068</t>
+  </si>
+  <si>
+    <t>T2-069</t>
+  </si>
+  <si>
+    <t>T2-070</t>
+  </si>
+  <si>
+    <t>T2-071</t>
+  </si>
+  <si>
+    <t>T2-072</t>
+  </si>
+  <si>
+    <t>T2-073</t>
+  </si>
+  <si>
+    <t>T2-074</t>
+  </si>
+  <si>
+    <t>T2-075</t>
+  </si>
+  <si>
+    <t>T2-076</t>
+  </si>
+  <si>
+    <t>T2-077</t>
+  </si>
+  <si>
+    <t>T2-078</t>
+  </si>
+  <si>
+    <t>T2-079</t>
+  </si>
+  <si>
+    <t>T2-080</t>
+  </si>
+  <si>
+    <t>T2-081</t>
+  </si>
+  <si>
+    <t>T2-082</t>
+  </si>
+  <si>
+    <t>T2-083</t>
+  </si>
+  <si>
+    <t>T2-084</t>
+  </si>
+  <si>
+    <t>T2-085</t>
+  </si>
+  <si>
+    <t>T2-086</t>
+  </si>
+  <si>
+    <t>T2-087</t>
+  </si>
+  <si>
+    <t>T2-088</t>
+  </si>
+  <si>
+    <t>T2-089</t>
+  </si>
+  <si>
+    <t>T2-090</t>
+  </si>
+  <si>
+    <t>T2-091</t>
+  </si>
+  <si>
+    <t>T2-092</t>
+  </si>
+  <si>
+    <t>T2-093</t>
+  </si>
+  <si>
+    <t>T2-094</t>
+  </si>
+  <si>
+    <t>T2-095</t>
+  </si>
+  <si>
+    <t>T2-096</t>
+  </si>
+  <si>
+    <t>T2-097</t>
+  </si>
+  <si>
+    <t>T2-098</t>
+  </si>
+  <si>
+    <t>T2-099</t>
+  </si>
+  <si>
+    <t>T2-100</t>
+  </si>
+  <si>
+    <t>T2-101</t>
+  </si>
+  <si>
+    <t>T2-102</t>
+  </si>
+  <si>
+    <t>T2-103</t>
+  </si>
+  <si>
+    <t>T2-105</t>
+  </si>
+  <si>
+    <t>T2-106</t>
+  </si>
+  <si>
+    <t>T2-107</t>
+  </si>
+  <si>
+    <t>T1-085</t>
+  </si>
+  <si>
+    <t>Tier 1 Operators
+Tier 1 Authentication Policy</t>
+  </si>
+  <si>
+    <t>Tier 1 Server Operators
+Tier 1 Operators
+Tier 1 Authentication Policy</t>
+  </si>
+  <si>
+    <t>Klist shows 4 hour TGT with Tier 1 Authentication Silo Policy Enforced</t>
+  </si>
+  <si>
+    <t>Allowed to login with Tier 2 EUD Authentication Silo Policy Enforced</t>
+  </si>
+  <si>
+    <t>Klist shows 6 hour TGT with Tier 2 Authentication Silo Policy Enforced</t>
+  </si>
+  <si>
+    <t>Allowed to login with Tier 2 Authentication Silo Policy Enforced</t>
+  </si>
+  <si>
+    <t>Tier 0 Server Operators
+Tier 0 Operators
+Tier 0 Authentication Policy</t>
+  </si>
+  <si>
+    <t>Domain Admins
+Tier 0 Operators
+Tier 0 Authentication Policy</t>
+  </si>
+  <si>
+    <t>Allowed to login with Tier 0 Authentication Policy Enforced</t>
+  </si>
+  <si>
+    <t>Denied login with Tier 0 Authentication Policy Enforced - Event ID 105</t>
+  </si>
+  <si>
+    <t>Allowed to login with Tier 1 Authentication Policy Enforced</t>
+  </si>
+  <si>
+    <t>T1-086</t>
+  </si>
+  <si>
+    <t>T1-087</t>
+  </si>
+  <si>
+    <t>Auth Silo - Tier 1 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>Auth Silo - Tier 1 Member Server - RDP</t>
+  </si>
+  <si>
+    <t>T0-084</t>
+  </si>
+  <si>
+    <t>T0-085</t>
+  </si>
+  <si>
+    <t>Auth Silo - Tier 2 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>Auth Silo - Tier 2 End-User Device - Interactive</t>
+  </si>
+  <si>
+    <t>T0-086</t>
+  </si>
+  <si>
+    <t>Auth Silo - Deny Tier 0 Member Server - RDP</t>
+  </si>
+  <si>
+    <t>Auth Silo - Deny Domain Controller - RDP</t>
+  </si>
+  <si>
+    <t>Auth Silo - Deny Tier 0 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>Auth Silo - Deny Tier 2 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>Auth Silo - End-User Device Outside Tier Model - Interactive</t>
+  </si>
+  <si>
+    <t>T1-088</t>
+  </si>
+  <si>
+    <t>T1-089</t>
+  </si>
+  <si>
+    <t>Denied login with Tier 1 Authentication Policy Enforced - Event ID 105</t>
+  </si>
+  <si>
+    <t>Auth Silo - Deny Tier 1 Member Server - RDP</t>
+  </si>
+  <si>
+    <t>Auth Silo - Deny Tier 1 PAW - Interactive</t>
+  </si>
+  <si>
+    <t>T2-108</t>
+  </si>
+  <si>
+    <t>T2-109</t>
+  </si>
+  <si>
+    <t>T2-110</t>
+  </si>
+  <si>
+    <t>T2-111</t>
+  </si>
+  <si>
+    <t>T2-112</t>
+  </si>
+  <si>
+    <t>T2-113</t>
+  </si>
+  <si>
+    <t>Denied login with Tier 2 Authentication Policy Enforced - Event ID 105</t>
+  </si>
+  <si>
+    <t>T2-114</t>
+  </si>
+  <si>
+    <t>T2-115</t>
+  </si>
+  <si>
+    <t>T2-116</t>
+  </si>
+  <si>
+    <t>T2-117</t>
+  </si>
+  <si>
+    <t>T2-118</t>
+  </si>
+  <si>
+    <t>OTM-043</t>
+  </si>
+  <si>
+    <t>OTM-044</t>
+  </si>
+  <si>
+    <t>OTM-045</t>
+  </si>
+  <si>
+    <t>OTM-046</t>
+  </si>
+  <si>
+    <t>Auth Silos</t>
+  </si>
+  <si>
+    <t>When testing auth silos ensure to remove the 5 URA Deny from the Tier Model Authentication GPOS (Tier 0/1/2 Servers/PAWs) to ensure URA are not denying and only Auth Silos are applying</t>
   </si>
 </sst>
 </file>
@@ -2995,7 +3362,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3075,14 +3442,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -3090,27 +3449,7 @@
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="122">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="130">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -3168,136 +3507,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3483,6 +3692,236 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3555,28 +3994,28 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -3606,28 +4045,28 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -3920,7 +4359,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BBDC83E0-955E-4441-8E62-48B5AD3B7F7C}" name="Table8" displayName="Table8" ref="A1:O42" totalsRowShown="0" headerRowDxfId="121" headerRowBorderDxfId="120" tableBorderDxfId="119">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BBDC83E0-955E-4441-8E62-48B5AD3B7F7C}" name="Table8" displayName="Table8" ref="A1:O42" totalsRowShown="0" headerRowDxfId="129" headerRowBorderDxfId="128" tableBorderDxfId="127">
   <autoFilter ref="A1:O42" xr:uid="{BBDC83E0-955E-4441-8E62-48B5AD3B7F7C}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{A4997F13-AC91-46E7-9C27-5D05D8995D60}" name="Test Num"/>
@@ -3930,13 +4369,13 @@
     <tableColumn id="5" xr3:uid="{1FC76C0A-9A26-4B06-8490-F200EC00E4EF}" name="Member Of"/>
     <tableColumn id="6" xr3:uid="{49812656-8701-4DCA-8B70-59D7F432AD83}" name="Test Device"/>
     <tableColumn id="7" xr3:uid="{2B963348-44AC-44ED-8F30-26C149C9F64D}" name="Steps"/>
-    <tableColumn id="8" xr3:uid="{0D06EF6C-0CD0-4677-876B-3995F790C765}" name="Result 1" dataDxfId="118"/>
-    <tableColumn id="9" xr3:uid="{0B8B0955-473B-49C5-8D3A-A400A4117CBE}" name="Date 1" dataDxfId="117" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{0F470D11-D265-4503-9506-43C538AE2DC1}" name="Tester 1" dataDxfId="116" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{0D06EF6C-0CD0-4677-876B-3995F790C765}" name="Result 1" dataDxfId="126"/>
+    <tableColumn id="9" xr3:uid="{0B8B0955-473B-49C5-8D3A-A400A4117CBE}" name="Date 1" dataDxfId="125" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{0F470D11-D265-4503-9506-43C538AE2DC1}" name="Tester 1" dataDxfId="124" dataCellStyle="Normal"/>
     <tableColumn id="11" xr3:uid="{228CBCFE-86F5-481F-BDEC-40B48BBE889D}" name="Comments 1" dataCellStyle="Normal"/>
-    <tableColumn id="12" xr3:uid="{E5EF96BB-126C-480C-B7FC-77C739DF5B1D}" name="Results 2" dataDxfId="115"/>
+    <tableColumn id="12" xr3:uid="{E5EF96BB-126C-480C-B7FC-77C739DF5B1D}" name="Results 2" dataDxfId="123"/>
     <tableColumn id="13" xr3:uid="{5DB34468-1538-4007-82D6-8EEA8A8C1993}" name="Date 2"/>
-    <tableColumn id="14" xr3:uid="{C18F0626-9D7E-4106-9931-B9986AADE4D0}" name="Tester 2" dataDxfId="114"/>
+    <tableColumn id="14" xr3:uid="{C18F0626-9D7E-4106-9931-B9986AADE4D0}" name="Tester 2" dataDxfId="122"/>
     <tableColumn id="15" xr3:uid="{0B0477E8-6A70-4B4D-B98E-D459B76D22C7}" name="Comments 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3944,96 +4383,96 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FFF45944-2A4D-4033-B755-D7B4507490C2}" name="Table4" displayName="Table4" ref="A1:O84" totalsRowShown="0" headerRowDxfId="113" dataDxfId="112">
-  <autoFilter ref="A1:O84" xr:uid="{FFF45944-2A4D-4033-B755-D7B4507490C2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FFF45944-2A4D-4033-B755-D7B4507490C2}" name="Table4" displayName="Table4" ref="A1:O87" totalsRowShown="0" headerRowDxfId="121" dataDxfId="120">
+  <autoFilter ref="A1:O87" xr:uid="{FFF45944-2A4D-4033-B755-D7B4507490C2}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{BE52AF1E-BE97-41AD-91ED-DE34C5EE886F}" name="Test Num" dataDxfId="111"/>
-    <tableColumn id="2" xr3:uid="{E7880774-D716-414F-B5F2-C108A070B2D5}" name="Role" dataDxfId="110"/>
-    <tableColumn id="3" xr3:uid="{76377402-3D21-45AB-A9F3-08B60FE18923}" name="Test Case" dataDxfId="109"/>
-    <tableColumn id="4" xr3:uid="{A9117327-F067-4E1B-BBDC-9C9DB8B27F70}" name="Account Tier" dataDxfId="108"/>
-    <tableColumn id="5" xr3:uid="{6FE7F356-C55D-4BD6-B12D-32030CF1EBB0}" name="Member Of" dataDxfId="107"/>
-    <tableColumn id="6" xr3:uid="{A2643D89-0009-48D0-97AD-D861219BCB64}" name="Test Device" dataDxfId="106"/>
-    <tableColumn id="7" xr3:uid="{2DF16A02-3509-4DC9-B46E-952EB6D09826}" name="Steps" dataDxfId="105"/>
-    <tableColumn id="15" xr3:uid="{D3B15A47-8060-4494-9BEC-6113C9237E7B}" name="Result 1" dataDxfId="104"/>
-    <tableColumn id="14" xr3:uid="{D468D462-294C-4B16-A0EC-BE7A78192C80}" name="Date 1" dataDxfId="103"/>
-    <tableColumn id="13" xr3:uid="{DFED3155-8A6F-4EFB-8E41-565AD7D0829E}" name="Tester 1" dataDxfId="102"/>
-    <tableColumn id="12" xr3:uid="{FA56428D-5B55-4936-B617-48C969D29555}" name="Comments 1" dataDxfId="101"/>
-    <tableColumn id="8" xr3:uid="{4AC14231-7F44-4F5A-8DCB-7352EBEF09BF}" name="Results 2" dataDxfId="100"/>
-    <tableColumn id="10" xr3:uid="{A13A5449-5099-47A4-917C-995C610284DC}" name="Date 2" dataDxfId="99"/>
-    <tableColumn id="11" xr3:uid="{2EA75155-8D1B-4327-AAEF-A34C76441CF5}" name="Tester 2" dataDxfId="98"/>
-    <tableColumn id="9" xr3:uid="{781068EC-2F0D-416E-BD14-653C89C646CF}" name="Comments 2" dataDxfId="97"/>
+    <tableColumn id="1" xr3:uid="{BE52AF1E-BE97-41AD-91ED-DE34C5EE886F}" name="Test Num" dataDxfId="119"/>
+    <tableColumn id="2" xr3:uid="{E7880774-D716-414F-B5F2-C108A070B2D5}" name="Role" dataDxfId="118"/>
+    <tableColumn id="3" xr3:uid="{76377402-3D21-45AB-A9F3-08B60FE18923}" name="Test Case" dataDxfId="117"/>
+    <tableColumn id="4" xr3:uid="{A9117327-F067-4E1B-BBDC-9C9DB8B27F70}" name="Account Tier" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{6FE7F356-C55D-4BD6-B12D-32030CF1EBB0}" name="Member Of" dataDxfId="115"/>
+    <tableColumn id="6" xr3:uid="{A2643D89-0009-48D0-97AD-D861219BCB64}" name="Test Device" dataDxfId="114"/>
+    <tableColumn id="7" xr3:uid="{2DF16A02-3509-4DC9-B46E-952EB6D09826}" name="Steps" dataDxfId="113"/>
+    <tableColumn id="15" xr3:uid="{D3B15A47-8060-4494-9BEC-6113C9237E7B}" name="Result 1" dataDxfId="112"/>
+    <tableColumn id="14" xr3:uid="{D468D462-294C-4B16-A0EC-BE7A78192C80}" name="Date 1" dataDxfId="111"/>
+    <tableColumn id="13" xr3:uid="{DFED3155-8A6F-4EFB-8E41-565AD7D0829E}" name="Tester 1" dataDxfId="110"/>
+    <tableColumn id="12" xr3:uid="{FA56428D-5B55-4936-B617-48C969D29555}" name="Comments 1" dataDxfId="109"/>
+    <tableColumn id="8" xr3:uid="{4AC14231-7F44-4F5A-8DCB-7352EBEF09BF}" name="Results 2" dataDxfId="108"/>
+    <tableColumn id="10" xr3:uid="{A13A5449-5099-47A4-917C-995C610284DC}" name="Date 2" dataDxfId="107"/>
+    <tableColumn id="11" xr3:uid="{2EA75155-8D1B-4327-AAEF-A34C76441CF5}" name="Tester 2" dataDxfId="106"/>
+    <tableColumn id="9" xr3:uid="{781068EC-2F0D-416E-BD14-653C89C646CF}" name="Comments 2" dataDxfId="105"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D1C8D22-8799-4789-AC90-A2DA43011B4B}" name="Table3" displayName="Table3" ref="A1:O86" totalsRowShown="0" headerRowDxfId="96" dataDxfId="95">
-  <autoFilter ref="A1:O86" xr:uid="{3D1C8D22-8799-4789-AC90-A2DA43011B4B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D1C8D22-8799-4789-AC90-A2DA43011B4B}" name="Table3" displayName="Table3" ref="A1:O90" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
+  <autoFilter ref="A1:O90" xr:uid="{3D1C8D22-8799-4789-AC90-A2DA43011B4B}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{D09E58BE-FEF9-41DE-9D8D-1DADA7CB1A3E}" name="Test Num" dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{7918EE24-0094-48F6-8ED5-8FB237D184F0}" name="Role" dataDxfId="93"/>
-    <tableColumn id="3" xr3:uid="{C7183E2C-E9B9-42AC-A164-5F1998E926CC}" name="Test Case" dataDxfId="92"/>
-    <tableColumn id="4" xr3:uid="{9C400D12-E338-4EFE-A7C1-92B5F198A30B}" name="Account Tier" dataDxfId="91"/>
-    <tableColumn id="5" xr3:uid="{9FB3EAFA-D413-4020-9923-30FBEA1C2483}" name="Member Of" dataDxfId="90"/>
-    <tableColumn id="6" xr3:uid="{1F963AD9-DBB5-44C8-BAC6-ADB071A246EC}" name="Test Device" dataDxfId="89"/>
-    <tableColumn id="7" xr3:uid="{961A93C3-EF44-4D30-BA51-3AB1F368149E}" name="Steps" dataDxfId="88"/>
-    <tableColumn id="15" xr3:uid="{64EBB73C-E234-4AEA-BF57-BA56C45781A4}" name="Result 1" dataDxfId="87"/>
-    <tableColumn id="14" xr3:uid="{57728B78-D8B9-469F-BE14-1F7300E25B0A}" name="Date 1" dataDxfId="86"/>
-    <tableColumn id="13" xr3:uid="{A85C0F5E-3B6E-49C0-B6F0-70D0979863B9}" name="Tester 1" dataDxfId="85"/>
-    <tableColumn id="12" xr3:uid="{4B38473F-A7B1-469C-A50C-01068E9ED7CE}" name="Comments 1" dataDxfId="84"/>
-    <tableColumn id="8" xr3:uid="{4F269C65-5B7E-456A-A494-D44AB144D363}" name="Results 2" dataDxfId="83"/>
-    <tableColumn id="10" xr3:uid="{2109691A-4EDC-458B-A336-6B6E190B9A92}" name="Date 2" dataDxfId="82"/>
-    <tableColumn id="11" xr3:uid="{930C7486-8059-4A94-8E80-E4541438DEB4}" name="Tester 2" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{4B6480AC-F6F9-44B9-8DA4-A907BB1A0276}" name="Comments 2" dataDxfId="80"/>
+    <tableColumn id="1" xr3:uid="{D09E58BE-FEF9-41DE-9D8D-1DADA7CB1A3E}" name="Test Num" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{7918EE24-0094-48F6-8ED5-8FB237D184F0}" name="Role" dataDxfId="101"/>
+    <tableColumn id="3" xr3:uid="{C7183E2C-E9B9-42AC-A164-5F1998E926CC}" name="Test Case" dataDxfId="100"/>
+    <tableColumn id="4" xr3:uid="{9C400D12-E338-4EFE-A7C1-92B5F198A30B}" name="Account Tier" dataDxfId="99"/>
+    <tableColumn id="5" xr3:uid="{9FB3EAFA-D413-4020-9923-30FBEA1C2483}" name="Member Of" dataDxfId="98"/>
+    <tableColumn id="6" xr3:uid="{1F963AD9-DBB5-44C8-BAC6-ADB071A246EC}" name="Test Device" dataDxfId="97"/>
+    <tableColumn id="7" xr3:uid="{961A93C3-EF44-4D30-BA51-3AB1F368149E}" name="Steps" dataDxfId="96"/>
+    <tableColumn id="15" xr3:uid="{64EBB73C-E234-4AEA-BF57-BA56C45781A4}" name="Result 1" dataDxfId="95"/>
+    <tableColumn id="14" xr3:uid="{57728B78-D8B9-469F-BE14-1F7300E25B0A}" name="Date 1" dataDxfId="94"/>
+    <tableColumn id="13" xr3:uid="{A85C0F5E-3B6E-49C0-B6F0-70D0979863B9}" name="Tester 1" dataDxfId="93"/>
+    <tableColumn id="12" xr3:uid="{4B38473F-A7B1-469C-A50C-01068E9ED7CE}" name="Comments 1" dataDxfId="92"/>
+    <tableColumn id="8" xr3:uid="{4F269C65-5B7E-456A-A494-D44AB144D363}" name="Results 2" dataDxfId="91"/>
+    <tableColumn id="10" xr3:uid="{2109691A-4EDC-458B-A336-6B6E190B9A92}" name="Date 2" dataDxfId="90"/>
+    <tableColumn id="11" xr3:uid="{930C7486-8059-4A94-8E80-E4541438DEB4}" name="Tester 2" dataDxfId="89"/>
+    <tableColumn id="9" xr3:uid="{4B6480AC-F6F9-44B9-8DA4-A907BB1A0276}" name="Comments 2" dataDxfId="88"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6CB453EC-9F38-4A1A-841E-12373A0046E8}" name="Table2" displayName="Table2" ref="A1:O108" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
-  <autoFilter ref="A1:O108" xr:uid="{6CB453EC-9F38-4A1A-841E-12373A0046E8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6CB453EC-9F38-4A1A-841E-12373A0046E8}" name="Table2" displayName="Table2" ref="A1:O118" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+  <autoFilter ref="A1:O118" xr:uid="{6CB453EC-9F38-4A1A-841E-12373A0046E8}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{6F968ADA-C366-45BB-8076-11A6E132598D}" name="Test Num" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{1CF9D31D-A3E8-43CB-9C53-1B5CA334451D}" name="Role" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{A4586D46-3561-4DB2-A5CD-82F11E112E36}" name="Test Case" dataDxfId="58"/>
-    <tableColumn id="4" xr3:uid="{3074E7FF-6671-4AF2-98D7-4B64EA286C21}" name="Account Tier" dataDxfId="57"/>
-    <tableColumn id="5" xr3:uid="{61DC852D-ACBB-4250-AE54-F784DBA0124F}" name="Member Of" dataDxfId="56"/>
-    <tableColumn id="6" xr3:uid="{A4A28542-1156-415C-B9A6-26B2C64571C8}" name="Test Device" dataDxfId="55"/>
-    <tableColumn id="7" xr3:uid="{508667C8-E7DC-4B36-B730-1BF07B072B26}" name="Steps" dataDxfId="54"/>
-    <tableColumn id="15" xr3:uid="{98B63D13-4B1B-4929-A507-3B339C9178DC}" name="Result 1" dataDxfId="53"/>
-    <tableColumn id="14" xr3:uid="{0960049F-6624-4EF2-A9BE-6C4BF1BF0B30}" name="Date 1" dataDxfId="52"/>
-    <tableColumn id="13" xr3:uid="{B8038056-A835-4C98-83D2-9F7F811DA5B5}" name="Tester 1" dataDxfId="51"/>
-    <tableColumn id="12" xr3:uid="{7A4FCB71-BD95-4A2A-9499-EE33978E1B72}" name="Comment 1" dataDxfId="50"/>
-    <tableColumn id="8" xr3:uid="{962A06FB-258E-4DB6-B7AD-C09A30D77672}" name="Results 2" dataDxfId="49"/>
-    <tableColumn id="10" xr3:uid="{385794D4-4829-4203-BE5E-17ECE94BC5D3}" name="Date 2" dataDxfId="48"/>
-    <tableColumn id="11" xr3:uid="{F0A1DEEA-8A69-45E5-9D9F-58AF6D63896D}" name="Tester 2" dataDxfId="47"/>
-    <tableColumn id="9" xr3:uid="{255C1446-C13E-4C8B-B25C-201918325FA2}" name="Comments 2" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{6F968ADA-C366-45BB-8076-11A6E132598D}" name="Test Num" dataDxfId="85"/>
+    <tableColumn id="2" xr3:uid="{1CF9D31D-A3E8-43CB-9C53-1B5CA334451D}" name="Role" dataDxfId="84"/>
+    <tableColumn id="3" xr3:uid="{A4586D46-3561-4DB2-A5CD-82F11E112E36}" name="Test Case" dataDxfId="83"/>
+    <tableColumn id="4" xr3:uid="{3074E7FF-6671-4AF2-98D7-4B64EA286C21}" name="Account Tier" dataDxfId="82"/>
+    <tableColumn id="5" xr3:uid="{61DC852D-ACBB-4250-AE54-F784DBA0124F}" name="Member Of" dataDxfId="81"/>
+    <tableColumn id="6" xr3:uid="{A4A28542-1156-415C-B9A6-26B2C64571C8}" name="Test Device" dataDxfId="80"/>
+    <tableColumn id="7" xr3:uid="{508667C8-E7DC-4B36-B730-1BF07B072B26}" name="Steps" dataDxfId="79"/>
+    <tableColumn id="15" xr3:uid="{98B63D13-4B1B-4929-A507-3B339C9178DC}" name="Result 1" dataDxfId="78"/>
+    <tableColumn id="14" xr3:uid="{0960049F-6624-4EF2-A9BE-6C4BF1BF0B30}" name="Date 1" dataDxfId="77"/>
+    <tableColumn id="13" xr3:uid="{B8038056-A835-4C98-83D2-9F7F811DA5B5}" name="Tester 1" dataDxfId="76"/>
+    <tableColumn id="12" xr3:uid="{7A4FCB71-BD95-4A2A-9499-EE33978E1B72}" name="Comment 1" dataDxfId="75"/>
+    <tableColumn id="8" xr3:uid="{962A06FB-258E-4DB6-B7AD-C09A30D77672}" name="Results 2" dataDxfId="74"/>
+    <tableColumn id="10" xr3:uid="{385794D4-4829-4203-BE5E-17ECE94BC5D3}" name="Date 2" dataDxfId="73"/>
+    <tableColumn id="11" xr3:uid="{F0A1DEEA-8A69-45E5-9D9F-58AF6D63896D}" name="Tester 2" dataDxfId="72"/>
+    <tableColumn id="9" xr3:uid="{255C1446-C13E-4C8B-B25C-201918325FA2}" name="Comments 2" dataDxfId="71"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EB17A5CC-E408-4C9A-B5B1-6D8E779BD4FF}" name="Table1" displayName="Table1" ref="A1:O42" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
-  <autoFilter ref="A1:O42" xr:uid="{EB17A5CC-E408-4C9A-B5B1-6D8E779BD4FF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EB17A5CC-E408-4C9A-B5B1-6D8E779BD4FF}" name="Table1" displayName="Table1" ref="A1:O46" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+  <autoFilter ref="A1:O46" xr:uid="{EB17A5CC-E408-4C9A-B5B1-6D8E779BD4FF}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{823BC357-BB93-4F33-BD5C-CA74E34526D5}" name="Test Num" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{17424961-31D2-4C05-8CB9-9657B47F8534}" name="Role" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{AF7EE82B-D8B0-461F-AC7A-26F79D6F1400}" name="Test Case" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{7C7C56AD-F058-48C0-B4E4-CCCAFF2251BB}" name="Account Tier" dataDxfId="74"/>
-    <tableColumn id="5" xr3:uid="{DED0F04D-B39D-4D1D-827C-FA435FA02FB5}" name="Member Of" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{89BD421D-B187-43BD-97FE-5DC073DE828B}" name="Test Device" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{A56500EF-650E-4E5B-8835-999502D63C09}" name="Steps" dataDxfId="71"/>
-    <tableColumn id="15" xr3:uid="{9EAAD511-E661-49CF-A644-79E3D2286F82}" name="Result 1" dataDxfId="70"/>
-    <tableColumn id="14" xr3:uid="{D147186E-F9DE-4DEE-AC48-717CF1F2EFFF}" name="Date 1" dataDxfId="69"/>
-    <tableColumn id="13" xr3:uid="{005F10CF-A98F-4680-A807-A3DA2AC11987}" name="Tester 1" dataDxfId="68"/>
-    <tableColumn id="12" xr3:uid="{B10B013E-B707-45F1-A349-E3949E0318B6}" name="Comments 1" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{B0760FD3-784D-4B94-9349-CCBCF60DDBDF}" name="Results 2" dataDxfId="66"/>
-    <tableColumn id="10" xr3:uid="{CF7BC678-11B8-4277-8A7D-BE27B1DD3883}" name="Date 2" dataDxfId="65"/>
-    <tableColumn id="11" xr3:uid="{E153E44B-CE3E-468C-BD29-0EC84853E492}" name="Tester 2" dataDxfId="64"/>
-    <tableColumn id="9" xr3:uid="{56D1854D-5874-4A46-8106-061E8E3D40DF}" name="Comments 2" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{823BC357-BB93-4F33-BD5C-CA74E34526D5}" name="Test Num" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{17424961-31D2-4C05-8CB9-9657B47F8534}" name="Role" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{AF7EE82B-D8B0-461F-AC7A-26F79D6F1400}" name="Test Case" dataDxfId="66"/>
+    <tableColumn id="4" xr3:uid="{7C7C56AD-F058-48C0-B4E4-CCCAFF2251BB}" name="Account Tier" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{DED0F04D-B39D-4D1D-827C-FA435FA02FB5}" name="Member Of" dataDxfId="64"/>
+    <tableColumn id="6" xr3:uid="{89BD421D-B187-43BD-97FE-5DC073DE828B}" name="Test Device" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{A56500EF-650E-4E5B-8835-999502D63C09}" name="Steps" dataDxfId="62"/>
+    <tableColumn id="15" xr3:uid="{9EAAD511-E661-49CF-A644-79E3D2286F82}" name="Result 1" dataDxfId="61"/>
+    <tableColumn id="14" xr3:uid="{D147186E-F9DE-4DEE-AC48-717CF1F2EFFF}" name="Date 1" dataDxfId="60"/>
+    <tableColumn id="13" xr3:uid="{005F10CF-A98F-4680-A807-A3DA2AC11987}" name="Tester 1" dataDxfId="59"/>
+    <tableColumn id="12" xr3:uid="{B10B013E-B707-45F1-A349-E3949E0318B6}" name="Comments 1" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{B0760FD3-784D-4B94-9349-CCBCF60DDBDF}" name="Results 2" dataDxfId="57"/>
+    <tableColumn id="10" xr3:uid="{CF7BC678-11B8-4277-8A7D-BE27B1DD3883}" name="Date 2" dataDxfId="56"/>
+    <tableColumn id="11" xr3:uid="{E153E44B-CE3E-468C-BD29-0EC84853E492}" name="Tester 2" dataDxfId="55"/>
+    <tableColumn id="9" xr3:uid="{56D1854D-5874-4A46-8106-061E8E3D40DF}" name="Comments 2" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4356,7 +4795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD685266-47A4-4775-B64D-76322AE37B32}">
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
@@ -4424,11 +4863,11 @@
       </c>
       <c r="I2" s="10">
         <f>COUNTIF(Deploy!H:H,"Pending")+COUNTIF('Tier 0'!H:H,"Pending")+COUNTIF('Tier 1'!H:H,"Pending")+COUNTIF('Tier 2'!H:H,"Pending")+COUNTIF('Outside TM'!H:H,"Pending")</f>
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="J2" s="10">
         <f>COUNTIF(Deploy!L:L,"Pending")+COUNTIF('Tier 0'!L:L,"Pending")+COUNTIF('Tier 1'!L:L,"Pending")+COUNTIF('Tier 2'!L:L,"Pending")+COUNTIF('Outside TM'!L:L,"Pending")</f>
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="K2" s="15">
         <f>SUM(I2:J2)</f>
@@ -4494,7 +4933,7 @@
       </c>
       <c r="I4" s="18">
         <f>COUNTIF(Deploy!H:H,"Pass")+COUNTIF('Tier 0'!H:H,"Pass")+COUNTIF('Tier 1'!H:H,"Pass")+COUNTIF('Tier 2'!H:H,"Pass")+COUNTIF('Outside TM'!H:H,"Pass")</f>
-        <v>335</v>
+        <v>378</v>
       </c>
       <c r="J4" s="18">
         <f>COUNTIF(Deploy!L:L,"Pass")+COUNTIF('Tier 0'!L:L,"Pass")+COUNTIF('Tier 1'!L:L,"Pass")+COUNTIF('Tier 2'!L:L,"Pass")+COUNTIF('Outside TM'!L:L,"Pass")</f>
@@ -4502,7 +4941,7 @@
       </c>
       <c r="K4" s="19">
         <f t="shared" si="0"/>
-        <v>561</v>
+        <v>604</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -4788,6 +5227,16 @@
       </c>
       <c r="B40" t="s">
         <v>773</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="24" x14ac:dyDescent="0.4">
+      <c r="A42" s="4" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>994</v>
       </c>
     </row>
   </sheetData>
@@ -4795,17 +5244,17 @@
     <mergeCell ref="A28:D28"/>
   </mergeCells>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="cellIs" dxfId="45" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="53" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3:K3">
-    <cfRule type="cellIs" dxfId="44" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4:K4">
-    <cfRule type="cellIs" dxfId="43" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="51" priority="1" operator="greaterThan">
       <formula>132</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5244,11 +5693,14 @@
       <c r="M10" s="8"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>862</v>
+      </c>
       <c r="B11" t="s">
         <v>663</v>
       </c>
       <c r="C11" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="D11" t="s">
         <v>88</v>
@@ -5260,12 +5712,14 @@
         <v>306</v>
       </c>
       <c r="G11" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="I11" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I11" s="8">
+        <v>46261</v>
+      </c>
       <c r="J11" s="7" t="s">
         <v>704</v>
       </c>
@@ -5275,6 +5729,9 @@
       <c r="M11" s="8"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>863</v>
+      </c>
       <c r="B12" t="s">
         <v>663</v>
       </c>
@@ -5313,6 +5770,9 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>864</v>
+      </c>
       <c r="B13" t="s">
         <v>663</v>
       </c>
@@ -5351,6 +5811,9 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>865</v>
+      </c>
       <c r="B14" t="s">
         <v>663</v>
       </c>
@@ -5389,6 +5852,9 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>866</v>
+      </c>
       <c r="B15" t="s">
         <v>663</v>
       </c>
@@ -5427,6 +5893,9 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>867</v>
+      </c>
       <c r="B16" t="s">
         <v>663</v>
       </c>
@@ -5464,7 +5933,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>868</v>
+      </c>
       <c r="B17" t="s">
         <v>663</v>
       </c>
@@ -5502,7 +5974,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>869</v>
+      </c>
       <c r="B18" t="s">
         <v>663</v>
       </c>
@@ -5535,7 +6010,10 @@
       </c>
       <c r="M18" s="8"/>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>870</v>
+      </c>
       <c r="B19" t="s">
         <v>663</v>
       </c>
@@ -5568,7 +6046,10 @@
       </c>
       <c r="M19" s="8"/>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>871</v>
+      </c>
       <c r="B20" t="s">
         <v>663</v>
       </c>
@@ -5601,7 +6082,10 @@
       </c>
       <c r="M20" s="8"/>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>872</v>
+      </c>
       <c r="B21" t="s">
         <v>663</v>
       </c>
@@ -5634,7 +6118,10 @@
       </c>
       <c r="M21" s="8"/>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>873</v>
+      </c>
       <c r="B22" t="s">
         <v>663</v>
       </c>
@@ -5667,12 +6154,15 @@
       </c>
       <c r="M22" s="8"/>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>874</v>
+      </c>
       <c r="B23" t="s">
         <v>663</v>
       </c>
       <c r="C23" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="D23" t="s">
         <v>88</v>
@@ -5684,22 +6174,26 @@
         <v>306</v>
       </c>
       <c r="G23" t="s">
-        <v>846</v>
-      </c>
-      <c r="H23" s="30" t="s">
+        <v>845</v>
+      </c>
+      <c r="H23" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I23" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="L23" s="20" t="s">
         <v>594</v>
       </c>
-      <c r="I23" s="32"/>
-      <c r="J23" s="7" t="s">
-        <v>704</v>
-      </c>
-      <c r="K23" s="31"/>
-      <c r="L23" s="30" t="s">
-        <v>594</v>
-      </c>
       <c r="M23" s="8"/>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>875</v>
+      </c>
       <c r="B24" t="s">
         <v>663</v>
       </c>
@@ -5737,7 +6231,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>876</v>
+      </c>
       <c r="B25" t="s">
         <v>716</v>
       </c>
@@ -5775,7 +6272,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>877</v>
+      </c>
       <c r="B26" t="s">
         <v>716</v>
       </c>
@@ -5808,7 +6308,10 @@
       </c>
       <c r="M26" s="8"/>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>878</v>
+      </c>
       <c r="B27" t="s">
         <v>716</v>
       </c>
@@ -5841,7 +6344,10 @@
       </c>
       <c r="M27" s="8"/>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>879</v>
+      </c>
       <c r="B28" t="s">
         <v>716</v>
       </c>
@@ -5874,12 +6380,15 @@
       </c>
       <c r="M28" s="8"/>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>880</v>
+      </c>
       <c r="B29" t="s">
         <v>716</v>
       </c>
       <c r="C29" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="D29" t="s">
         <v>88</v>
@@ -5891,12 +6400,14 @@
         <v>306</v>
       </c>
       <c r="G29" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="H29" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="I29" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I29" s="8">
+        <v>46261</v>
+      </c>
       <c r="J29" s="7" t="s">
         <v>704</v>
       </c>
@@ -5905,7 +6416,10 @@
       </c>
       <c r="M29" s="8"/>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>881</v>
+      </c>
       <c r="B30" t="s">
         <v>716</v>
       </c>
@@ -5943,7 +6457,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>882</v>
+      </c>
       <c r="B31" t="s">
         <v>716</v>
       </c>
@@ -5981,7 +6498,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>883</v>
+      </c>
       <c r="B32" t="s">
         <v>716</v>
       </c>
@@ -6019,7 +6539,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>884</v>
+      </c>
       <c r="B33" t="s">
         <v>716</v>
       </c>
@@ -6057,7 +6580,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>885</v>
+      </c>
       <c r="B34" t="s">
         <v>716</v>
       </c>
@@ -6095,7 +6621,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>886</v>
+      </c>
       <c r="B35" t="s">
         <v>716</v>
       </c>
@@ -6133,7 +6662,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>887</v>
+      </c>
       <c r="B36" t="s">
         <v>716</v>
       </c>
@@ -6166,7 +6698,10 @@
       </c>
       <c r="M36" s="8"/>
     </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>888</v>
+      </c>
       <c r="B37" t="s">
         <v>716</v>
       </c>
@@ -6199,7 +6734,10 @@
       </c>
       <c r="M37" s="8"/>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>889</v>
+      </c>
       <c r="B38" t="s">
         <v>716</v>
       </c>
@@ -6232,7 +6770,10 @@
       </c>
       <c r="M38" s="8"/>
     </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>890</v>
+      </c>
       <c r="B39" t="s">
         <v>716</v>
       </c>
@@ -6265,12 +6806,15 @@
       </c>
       <c r="M39" s="8"/>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>891</v>
+      </c>
       <c r="B40" t="s">
         <v>716</v>
       </c>
       <c r="C40" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="D40" t="s">
         <v>88</v>
@@ -6298,12 +6842,15 @@
       </c>
       <c r="M40" s="8"/>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>892</v>
+      </c>
       <c r="B41" t="s">
         <v>716</v>
       </c>
       <c r="C41" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="D41" t="s">
         <v>88</v>
@@ -6315,12 +6862,14 @@
         <v>306</v>
       </c>
       <c r="G41" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="H41" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="I41" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I41" s="8">
+        <v>46261</v>
+      </c>
       <c r="J41" s="7" t="s">
         <v>704</v>
       </c>
@@ -6329,7 +6878,10 @@
       </c>
       <c r="M41" s="8"/>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>893</v>
+      </c>
       <c r="B42" t="s">
         <v>716</v>
       </c>
@@ -6369,22 +6921,22 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H42 L2:L42">
-    <cfRule type="containsText" dxfId="42" priority="4" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="L2:L42 H2:H42">
+    <cfRule type="containsText" dxfId="50" priority="4" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="41" priority="5" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="49" priority="5" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="6" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="48" priority="6" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1:N1">
-    <cfRule type="containsText" dxfId="39" priority="7" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="47" priority="7" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="8" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="46" priority="8" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6409,14 +6961,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E517463F-4768-4C11-8EFB-DDC08B1B118E}">
-  <dimension ref="A1:O84"/>
+  <dimension ref="A1:O87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="58.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="64.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -9601,32 +10153,34 @@
       <c r="M77" s="8"/>
       <c r="O77" s="5"/>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>833</v>
+        <v>894</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>92</v>
+        <v>897</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>95</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>874</v>
+        <v>955</v>
       </c>
       <c r="H78" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I78" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I78" s="8">
+        <v>46261</v>
+      </c>
       <c r="J78" s="5" t="s">
         <v>704</v>
       </c>
@@ -9637,32 +10191,34 @@
       <c r="M78" s="8"/>
       <c r="O78" s="5"/>
     </row>
-    <row r="79" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>201</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>205</v>
+        <v>953</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>874</v>
+        <v>955</v>
       </c>
       <c r="H79" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I79" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I79" s="8">
+        <v>46261</v>
+      </c>
       <c r="J79" s="5" t="s">
         <v>704</v>
       </c>
@@ -9673,32 +10229,34 @@
       <c r="M79" s="8"/>
       <c r="O79" s="5"/>
     </row>
-    <row r="80" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>201</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>205</v>
+        <v>953</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>874</v>
+        <v>955</v>
       </c>
       <c r="H80" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I80" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I80" s="8">
+        <v>46261</v>
+      </c>
       <c r="J80" s="5" t="s">
         <v>704</v>
       </c>
@@ -9709,32 +10267,34 @@
       <c r="M80" s="8"/>
       <c r="O80" s="5"/>
     </row>
-    <row r="81" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>243</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>391</v>
+        <v>954</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>306</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>874</v>
+        <v>955</v>
       </c>
       <c r="H81" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I81" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I81" s="8">
+        <v>46261</v>
+      </c>
       <c r="J81" s="5" t="s">
         <v>704</v>
       </c>
@@ -9745,32 +10305,34 @@
       <c r="M81" s="8"/>
       <c r="O81" s="5"/>
     </row>
-    <row r="82" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>243</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>391</v>
+        <v>954</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>306</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>874</v>
+        <v>955</v>
       </c>
       <c r="H82" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I82" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I82" s="8">
+        <v>46261</v>
+      </c>
       <c r="J82" s="5" t="s">
         <v>704</v>
       </c>
@@ -9781,32 +10343,34 @@
       <c r="M82" s="8"/>
       <c r="O82" s="5"/>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>15</v>
+        <v>243</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>838</v>
+        <v>960</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>92</v>
+        <v>954</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>316</v>
+        <v>112</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>875</v>
+        <v>956</v>
       </c>
       <c r="H83" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I83" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I83" s="8">
+        <v>46261</v>
+      </c>
       <c r="J83" s="5" t="s">
         <v>704</v>
       </c>
@@ -9817,32 +10381,34 @@
       <c r="M83" s="8"/>
       <c r="O83" s="5"/>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>15</v>
+        <v>243</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>862</v>
+        <v>961</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>92</v>
+        <v>954</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>95</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>864</v>
+        <v>956</v>
       </c>
       <c r="H84" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I84" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I84" s="8">
+        <v>46261</v>
+      </c>
       <c r="J84" s="5" t="s">
         <v>704</v>
       </c>
@@ -9853,20 +10419,134 @@
       <c r="M84" s="8"/>
       <c r="O84" s="5"/>
     </row>
+    <row r="85" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A85" s="1" t="s">
+        <v>962</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>964</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>954</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>956</v>
+      </c>
+      <c r="H85" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I85" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J85" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K85" s="5"/>
+      <c r="L85" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M85" s="8"/>
+      <c r="O85" s="5"/>
+    </row>
+    <row r="86" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
+        <v>963</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>954</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>956</v>
+      </c>
+      <c r="H86" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I86" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J86" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K86" s="5"/>
+      <c r="L86" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M86" s="8"/>
+      <c r="O86" s="5"/>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A87" s="1" t="s">
+        <v>966</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="H87" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I87" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J87" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K87" s="5"/>
+      <c r="L87" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M87" s="8"/>
+      <c r="O87" s="5"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="L1:N1 L85:N1048576 H2:H84 L2:L84">
-    <cfRule type="containsText" dxfId="37" priority="7" operator="containsText" text="Fail">
+  <conditionalFormatting sqref="L1:N1 L88:N1048576 L2:L87 H2:H87">
+    <cfRule type="containsText" dxfId="45" priority="7" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H84 L2:L84">
-    <cfRule type="containsText" dxfId="36" priority="4" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="L2:L87 H2:H87">
+    <cfRule type="containsText" dxfId="44" priority="4" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1:N1 L85:N1048576 H2:H84 L2:L84">
-    <cfRule type="containsText" dxfId="35" priority="8" operator="containsText" text="Pass">
+  <conditionalFormatting sqref="L1:N1 L88:N1048576 L2:L87 H2:H87">
+    <cfRule type="containsText" dxfId="43" priority="8" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9881,7 +10561,7 @@
           <x14:formula1>
             <xm:f>Dropdown!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L84 H2:H84</xm:sqref>
+          <xm:sqref>H2:H87 L2:L87</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -9891,15 +10571,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F53C3A6B-E44E-43DD-8CFE-F822FAE3F5E1}">
-  <dimension ref="A1:O86"/>
+  <dimension ref="A1:O90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="71.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.28515625" style="5" bestFit="1" customWidth="1"/>
@@ -13168,32 +13848,34 @@
       </c>
       <c r="M81" s="8"/>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>854</v>
+        <v>895</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E82" s="1" t="s">
-        <v>137</v>
+      <c r="E82" s="2" t="s">
+        <v>947</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>112</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>872</v>
+        <v>957</v>
       </c>
       <c r="H82" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I82" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I82" s="8">
+        <v>46261</v>
+      </c>
       <c r="J82" s="5" t="s">
         <v>704</v>
       </c>
@@ -13202,32 +13884,34 @@
       </c>
       <c r="M82" s="8"/>
     </row>
-    <row r="83" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>201</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>89</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>206</v>
+        <v>948</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>112</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>872</v>
+        <v>957</v>
       </c>
       <c r="H83" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I83" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I83" s="8">
+        <v>46261</v>
+      </c>
       <c r="J83" s="5" t="s">
         <v>704</v>
       </c>
@@ -13236,32 +13920,34 @@
       </c>
       <c r="M83" s="8"/>
     </row>
-    <row r="84" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>201</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>89</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>206</v>
+        <v>948</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>112</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>872</v>
+        <v>957</v>
       </c>
       <c r="H84" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I84" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I84" s="8">
+        <v>46261</v>
+      </c>
       <c r="J84" s="5" t="s">
         <v>704</v>
       </c>
@@ -13270,32 +13956,34 @@
       </c>
       <c r="M84" s="8"/>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>15</v>
+        <v>201</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>838</v>
+        <v>968</v>
       </c>
       <c r="D85" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E85" s="1" t="s">
-        <v>137</v>
+      <c r="E85" s="2" t="s">
+        <v>948</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>316</v>
+        <v>112</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>873</v>
+        <v>957</v>
       </c>
       <c r="H85" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I85" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I85" s="8">
+        <v>46261</v>
+      </c>
       <c r="J85" s="5" t="s">
         <v>704</v>
       </c>
@@ -13304,29 +13992,34 @@
       </c>
       <c r="M85" s="8"/>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
+        <v>946</v>
+      </c>
       <c r="B86" s="1" t="s">
-        <v>15</v>
+        <v>201</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>862</v>
+        <v>967</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E86" s="1" t="s">
-        <v>137</v>
+      <c r="E86" s="2" t="s">
+        <v>948</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>112</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>863</v>
+        <v>957</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I86" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I86" s="8">
+        <v>46261</v>
+      </c>
       <c r="J86" s="5" t="s">
         <v>704</v>
       </c>
@@ -13335,55 +14028,186 @@
       </c>
       <c r="M86" s="8"/>
     </row>
+    <row r="87" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A87" s="1" t="s">
+        <v>958</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>969</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>948</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="H87" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I87" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J87" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L87" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M87" s="8"/>
+    </row>
+    <row r="88" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A88" s="1" t="s">
+        <v>959</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>970</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>947</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="H88" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I88" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J88" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L88" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M88" s="8"/>
+    </row>
+    <row r="89" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A89" s="1" t="s">
+        <v>972</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>947</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="H89" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I89" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J89" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L89" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M89" s="8"/>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A90" s="1" t="s">
+        <v>973</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>949</v>
+      </c>
+      <c r="H90" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I90" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J90" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L90" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M90" s="8"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H85">
-    <cfRule type="containsText" dxfId="34" priority="4" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="H2:H87 H89:H90 L2:L90">
+    <cfRule type="containsText" dxfId="42" priority="4" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="33" priority="5" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="41" priority="5" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="6" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="40" priority="6" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1:N1 L2:L85">
-    <cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="Fail">
+  <conditionalFormatting sqref="L1:N1">
+    <cfRule type="containsText" dxfId="39" priority="11" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L85">
-    <cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",L2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L1:N1 L2:L85">
-    <cfRule type="containsText" dxfId="29" priority="9" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="38" priority="12" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L87:N1048576">
-    <cfRule type="containsText" dxfId="28" priority="10" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",L87)))</formula>
+  <conditionalFormatting sqref="L91:N1048576">
+    <cfRule type="containsText" dxfId="37" priority="13" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",L91)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="27" priority="11" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",L87)))</formula>
+    <cfRule type="containsText" dxfId="36" priority="14" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",L91)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86 L86">
-    <cfRule type="containsText" dxfId="26" priority="2" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H86)))</formula>
+  <conditionalFormatting sqref="H88">
+    <cfRule type="containsText" dxfId="35" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H88)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86 L86">
-    <cfRule type="containsText" dxfId="25" priority="1" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H86)))</formula>
+  <conditionalFormatting sqref="H88">
+    <cfRule type="containsText" dxfId="34" priority="1" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H88)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86 L86">
-    <cfRule type="containsText" dxfId="24" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H86)))</formula>
+  <conditionalFormatting sqref="H88">
+    <cfRule type="containsText" dxfId="33" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H88)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13397,7 +14221,7 @@
           <x14:formula1>
             <xm:f>Dropdown!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H86 L2:L86</xm:sqref>
+          <xm:sqref>L2:L89 L90 H2:H89 H90</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -13407,7 +14231,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587115D9-8AB9-43C8-B333-F088A3B3F9B4}">
-  <dimension ref="A1:O108"/>
+  <dimension ref="A1:O118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -15974,6 +16798,9 @@
       </c>
     </row>
     <row r="63" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>901</v>
+      </c>
       <c r="B63" s="1" t="s">
         <v>127</v>
       </c>
@@ -15992,18 +16819,26 @@
       <c r="G63" s="2" t="s">
         <v>832</v>
       </c>
-      <c r="H63" s="6" t="s">
+      <c r="H63" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I63" s="8">
+        <v>46072</v>
+      </c>
+      <c r="J63" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K63" s="6"/>
+      <c r="L63" s="5" t="s">
         <v>594</v>
       </c>
-      <c r="I63" s="29"/>
-      <c r="J63" s="5" t="s">
-        <v>704</v>
-      </c>
-      <c r="K63" s="6"/>
       <c r="M63" s="27"/>
       <c r="N63" s="7"/>
     </row>
     <row r="64" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>902</v>
+      </c>
       <c r="B64" s="1" t="s">
         <v>479</v>
       </c>
@@ -16042,7 +16877,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="65" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>903</v>
+      </c>
       <c r="B65" s="1" t="s">
         <v>47</v>
       </c>
@@ -16080,7 +16918,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="66" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>904</v>
+      </c>
       <c r="B66" s="1" t="s">
         <v>47</v>
       </c>
@@ -16118,7 +16959,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="67" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>905</v>
+      </c>
       <c r="B67" s="1" t="s">
         <v>47</v>
       </c>
@@ -16156,7 +17000,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="68" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>906</v>
+      </c>
       <c r="B68" s="1" t="s">
         <v>47</v>
       </c>
@@ -16195,7 +17042,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="69" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>907</v>
+      </c>
       <c r="B69" s="1" t="s">
         <v>47</v>
       </c>
@@ -16234,7 +17084,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="70" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>908</v>
+      </c>
       <c r="B70" s="1" t="s">
         <v>47</v>
       </c>
@@ -16272,7 +17125,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="71" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>909</v>
+      </c>
       <c r="B71" s="1" t="s">
         <v>47</v>
       </c>
@@ -16310,7 +17166,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="72" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>910</v>
+      </c>
       <c r="B72" s="1" t="s">
         <v>47</v>
       </c>
@@ -16348,7 +17207,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="73" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>911</v>
+      </c>
       <c r="B73" s="1" t="s">
         <v>47</v>
       </c>
@@ -16386,7 +17248,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="74" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>912</v>
+      </c>
       <c r="B74" s="1" t="s">
         <v>47</v>
       </c>
@@ -16424,7 +17289,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="75" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>913</v>
+      </c>
       <c r="B75" s="1" t="s">
         <v>47</v>
       </c>
@@ -16462,7 +17330,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="76" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>914</v>
+      </c>
       <c r="B76" s="1" t="s">
         <v>47</v>
       </c>
@@ -16500,7 +17371,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="77" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>915</v>
+      </c>
       <c r="B77" s="1" t="s">
         <v>47</v>
       </c>
@@ -16538,7 +17412,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="78" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>916</v>
+      </c>
       <c r="B78" s="1" t="s">
         <v>47</v>
       </c>
@@ -16576,7 +17453,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="79" spans="2:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>917</v>
+      </c>
       <c r="B79" s="1" t="s">
         <v>47</v>
       </c>
@@ -16614,7 +17494,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>918</v>
+      </c>
       <c r="B80" s="1" t="s">
         <v>212</v>
       </c>
@@ -16652,7 +17535,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="81" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>919</v>
+      </c>
       <c r="B81" s="1" t="s">
         <v>25</v>
       </c>
@@ -16687,7 +17573,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="82" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A82" s="1" t="s">
+        <v>920</v>
+      </c>
       <c r="B82" s="1" t="s">
         <v>72</v>
       </c>
@@ -16722,7 +17611,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="83" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A83" s="1" t="s">
+        <v>921</v>
+      </c>
       <c r="B83" s="1" t="s">
         <v>72</v>
       </c>
@@ -16757,7 +17649,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="84" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A84" s="1" t="s">
+        <v>922</v>
+      </c>
       <c r="B84" s="1" t="s">
         <v>72</v>
       </c>
@@ -16793,7 +17688,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="85" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A85" s="1" t="s">
+        <v>923</v>
+      </c>
       <c r="B85" s="1" t="s">
         <v>15</v>
       </c>
@@ -16828,7 +17726,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="86" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
+        <v>924</v>
+      </c>
       <c r="B86" s="1" t="s">
         <v>15</v>
       </c>
@@ -16863,7 +17764,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="87" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A87" s="1" t="s">
+        <v>925</v>
+      </c>
       <c r="B87" s="1" t="s">
         <v>15</v>
       </c>
@@ -16899,7 +17803,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="88" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A88" s="1" t="s">
+        <v>926</v>
+      </c>
       <c r="B88" s="1" t="s">
         <v>119</v>
       </c>
@@ -16937,7 +17844,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="89" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A89" s="1" t="s">
+        <v>927</v>
+      </c>
       <c r="B89" s="1" t="s">
         <v>119</v>
       </c>
@@ -16975,7 +17885,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="90" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A90" s="1" t="s">
+        <v>928</v>
+      </c>
       <c r="B90" s="1" t="s">
         <v>72</v>
       </c>
@@ -17013,7 +17926,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="91" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A91" s="1" t="s">
+        <v>929</v>
+      </c>
       <c r="B91" s="1" t="s">
         <v>72</v>
       </c>
@@ -17051,7 +17967,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="92" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A92" s="1" t="s">
+        <v>930</v>
+      </c>
       <c r="B92" s="1" t="s">
         <v>332</v>
       </c>
@@ -17086,7 +18005,10 @@
         <v>706</v>
       </c>
     </row>
-    <row r="93" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A93" s="1" t="s">
+        <v>931</v>
+      </c>
       <c r="B93" s="1" t="s">
         <v>357</v>
       </c>
@@ -17125,7 +18047,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="94" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A94" s="1" t="s">
+        <v>932</v>
+      </c>
       <c r="B94" s="1" t="s">
         <v>332</v>
       </c>
@@ -17164,7 +18089,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="95" spans="2:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A95" s="1" t="s">
+        <v>933</v>
+      </c>
       <c r="B95" s="1" t="s">
         <v>332</v>
       </c>
@@ -17203,7 +18131,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="96" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A96" s="1" t="s">
+        <v>934</v>
+      </c>
       <c r="B96" s="1" t="s">
         <v>72</v>
       </c>
@@ -17242,7 +18173,10 @@
         <v>705</v>
       </c>
     </row>
-    <row r="97" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A97" s="1" t="s">
+        <v>935</v>
+      </c>
       <c r="B97" s="1" t="s">
         <v>72</v>
       </c>
@@ -17282,7 +18216,10 @@
       </c>
       <c r="O97" s="7"/>
     </row>
-    <row r="98" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A98" s="1" t="s">
+        <v>936</v>
+      </c>
       <c r="B98" s="1" t="s">
         <v>25</v>
       </c>
@@ -17322,7 +18259,10 @@
       </c>
       <c r="O98" s="7"/>
     </row>
-    <row r="99" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A99" s="1" t="s">
+        <v>937</v>
+      </c>
       <c r="B99" s="1" t="s">
         <v>292</v>
       </c>
@@ -17362,7 +18302,10 @@
       </c>
       <c r="O99" s="7"/>
     </row>
-    <row r="100" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A100" s="1" t="s">
+        <v>938</v>
+      </c>
       <c r="B100" s="1" t="s">
         <v>72</v>
       </c>
@@ -17397,7 +18340,10 @@
       <c r="M100" s="27"/>
       <c r="N100" s="7"/>
     </row>
-    <row r="101" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A101" s="1" t="s">
+        <v>939</v>
+      </c>
       <c r="B101" s="1" t="s">
         <v>72</v>
       </c>
@@ -17432,7 +18378,10 @@
       <c r="M101" s="27"/>
       <c r="N101" s="7"/>
     </row>
-    <row r="102" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A102" s="1" t="s">
+        <v>940</v>
+      </c>
       <c r="B102" s="1" t="s">
         <v>25</v>
       </c>
@@ -17467,7 +18416,10 @@
       <c r="M102" s="27"/>
       <c r="N102" s="7"/>
     </row>
-    <row r="103" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A103" s="1" t="s">
+        <v>941</v>
+      </c>
       <c r="B103" s="1" t="s">
         <v>25</v>
       </c>
@@ -17502,29 +18454,34 @@
       <c r="M103" s="27"/>
       <c r="N103" s="7"/>
     </row>
-    <row r="104" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A104" s="1" t="s">
+        <v>942</v>
+      </c>
       <c r="B104" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>865</v>
+        <v>896</v>
       </c>
       <c r="D104" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E104" s="1" t="s">
-        <v>5</v>
+      <c r="E104" s="2" t="s">
+        <v>899</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G104" s="1" t="s">
-        <v>871</v>
+        <v>952</v>
       </c>
       <c r="H104" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I104" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I104" s="8">
+        <v>46261</v>
+      </c>
       <c r="J104" s="5" t="s">
         <v>704</v>
       </c>
@@ -17534,29 +18491,34 @@
       <c r="M104" s="27"/>
       <c r="N104" s="7"/>
     </row>
-    <row r="105" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A105" s="1" t="s">
+        <v>943</v>
+      </c>
       <c r="B105" s="1" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>838</v>
+        <v>861</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E105" s="1" t="s">
-        <v>5</v>
+      <c r="E105" s="2" t="s">
+        <v>900</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>870</v>
+        <v>950</v>
       </c>
       <c r="H105" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I105" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I105" s="8">
+        <v>46261</v>
+      </c>
       <c r="J105" s="5" t="s">
         <v>704</v>
       </c>
@@ -17566,170 +18528,556 @@
       <c r="M105" s="27"/>
       <c r="N105" s="7"/>
     </row>
-    <row r="106" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A106" s="1" t="s">
+        <v>944</v>
+      </c>
       <c r="B106" s="1" t="s">
-        <v>15</v>
+        <v>332</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="D106" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>92</v>
+        <v>333</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>7</v>
+        <v>315</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>866</v>
+        <v>950</v>
       </c>
       <c r="H106" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I106" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I106" s="8">
+        <v>46261</v>
+      </c>
       <c r="J106" s="5" t="s">
         <v>704</v>
       </c>
+      <c r="K106" s="6"/>
       <c r="L106" s="5" t="s">
         <v>594</v>
       </c>
       <c r="M106" s="27"/>
       <c r="N106" s="7"/>
     </row>
-    <row r="107" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A107" s="1" t="s">
+        <v>945</v>
+      </c>
       <c r="B107" s="1" t="s">
-        <v>332</v>
+        <v>15</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>867</v>
+        <v>968</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="E107" s="1" t="s">
-        <v>333</v>
+        <v>3</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>899</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>315</v>
+        <v>7</v>
       </c>
       <c r="G107" s="1" t="s">
-        <v>869</v>
+        <v>983</v>
       </c>
       <c r="H107" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I107" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I107" s="8">
+        <v>46261</v>
+      </c>
       <c r="J107" s="5" t="s">
         <v>704</v>
       </c>
+      <c r="K107" s="6"/>
       <c r="L107" s="5" t="s">
         <v>594</v>
       </c>
       <c r="M107" s="27"/>
       <c r="N107" s="7"/>
     </row>
-    <row r="108" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A108" s="1" t="s">
+        <v>977</v>
+      </c>
       <c r="B108" s="1" t="s">
-        <v>332</v>
+        <v>15</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>838</v>
+        <v>967</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="E108" s="1" t="s">
-        <v>333</v>
+        <v>3</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>899</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>316</v>
+        <v>7</v>
       </c>
       <c r="G108" s="1" t="s">
-        <v>868</v>
+        <v>983</v>
       </c>
       <c r="H108" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="I108" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="I108" s="8">
+        <v>46261</v>
+      </c>
       <c r="J108" s="5" t="s">
         <v>704</v>
       </c>
+      <c r="K108" s="6"/>
       <c r="L108" s="5" t="s">
         <v>594</v>
       </c>
       <c r="M108" s="27"/>
       <c r="N108" s="7"/>
     </row>
+    <row r="109" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A109" s="1" t="s">
+        <v>978</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>969</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H109" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I109" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J109" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K109" s="6"/>
+      <c r="L109" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M109" s="27"/>
+      <c r="N109" s="7"/>
+    </row>
+    <row r="110" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A110" s="1" t="s">
+        <v>979</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>967</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H110" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I110" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J110" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K110" s="6"/>
+      <c r="L110" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M110" s="27"/>
+      <c r="N110" s="7"/>
+    </row>
+    <row r="111" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A111" s="1" t="s">
+        <v>980</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>969</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H111" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I111" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J111" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K111" s="6"/>
+      <c r="L111" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M111" s="27"/>
+      <c r="N111" s="7"/>
+    </row>
+    <row r="112" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A112" s="1" t="s">
+        <v>981</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>975</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H112" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I112" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J112" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K112" s="6"/>
+      <c r="L112" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M112" s="27"/>
+      <c r="N112" s="7"/>
+    </row>
+    <row r="113" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A113" s="1" t="s">
+        <v>982</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>976</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H113" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I113" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J113" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K113" s="6"/>
+      <c r="L113" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M113" s="27"/>
+      <c r="N113" s="7"/>
+    </row>
+    <row r="114" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A114" s="1" t="s">
+        <v>984</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>975</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>900</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H114" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I114" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J114" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K114" s="6"/>
+      <c r="L114" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M114" s="27"/>
+      <c r="N114" s="7"/>
+    </row>
+    <row r="115" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A115" s="1" t="s">
+        <v>985</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>976</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H115" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I115" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J115" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K115" s="6"/>
+      <c r="L115" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M115" s="27"/>
+      <c r="N115" s="7"/>
+    </row>
+    <row r="116" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A116" s="1" t="s">
+        <v>986</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>970</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H116" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I116" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J116" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K116" s="6"/>
+      <c r="L116" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M116" s="27"/>
+      <c r="N116" s="7"/>
+    </row>
+    <row r="117" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A117" s="1" t="s">
+        <v>987</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H117" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I117" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J117" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="K117" s="6"/>
+      <c r="L117" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M117" s="27"/>
+      <c r="N117" s="7"/>
+    </row>
+    <row r="118" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A118" s="1" t="s">
+        <v>988</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>951</v>
+      </c>
+      <c r="H118" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I118" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J118" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L118" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="M118" s="27"/>
+      <c r="N118" s="7"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H103 L2:L103">
-    <cfRule type="containsText" dxfId="23" priority="13" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="L2:L118 H2:H118">
+    <cfRule type="containsText" dxfId="32" priority="7" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="14" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="15" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="30" priority="9" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1:N1">
-    <cfRule type="containsText" dxfId="20" priority="17" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="29" priority="23" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="18" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="28" priority="24" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L109:N1048576">
-    <cfRule type="containsText" dxfId="18" priority="29" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",L109)))</formula>
+  <conditionalFormatting sqref="L119:N1048576">
+    <cfRule type="containsText" dxfId="27" priority="35" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",L119)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="30" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",L109)))</formula>
+    <cfRule type="containsText" dxfId="26" priority="36" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",L119)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H104">
-    <cfRule type="containsText" dxfId="16" priority="4" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H104)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="5" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H104)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="6" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H104)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L104">
-    <cfRule type="containsText" dxfId="13" priority="8" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",L104)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L104">
-    <cfRule type="containsText" dxfId="12" priority="7" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",L104)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L104">
-    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",L104)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H105:H108 L105:L108">
-    <cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="Fail">
+  <conditionalFormatting sqref="H105 H107:H116">
+    <cfRule type="containsText" dxfId="25" priority="5" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H105)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H105:H108 L105:L108">
-    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="H105 H107:H116">
+    <cfRule type="containsText" dxfId="24" priority="4" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H105)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H105:H108 L105:L108">
-    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="Pass">
+  <conditionalFormatting sqref="H105 H107:H116">
+    <cfRule type="containsText" dxfId="23" priority="6" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H105)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H117:H118">
+    <cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H117)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H117:H118">
+    <cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H117)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H117:H118">
+    <cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H117)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17743,7 +19091,7 @@
           <x14:formula1>
             <xm:f>Dropdown!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L108 H2:H108</xm:sqref>
+          <xm:sqref>H2:H117 H118 L2:L117 L118</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -17753,16 +19101,16 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D99589B0-FA3B-4812-885A-F9A38E7B8BFD}">
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="41.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="62" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
@@ -19427,40 +20775,232 @@
         <v>706</v>
       </c>
     </row>
+    <row r="43" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>971</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>897</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>956</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I43" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J43" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L43" s="5" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>990</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>971</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>947</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I44" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L44" s="5" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>991</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I45" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L45" s="5" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>992</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>900</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="I46" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="L46" s="5" t="s">
+        <v>594</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="H2:H42">
-    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="Pending">
+    <cfRule type="containsText" dxfId="19" priority="13" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="18" priority="14" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="17" priority="15" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L42 L1:N1">
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Fail">
+  <conditionalFormatting sqref="L1:N1 L2:L42">
+    <cfRule type="containsText" dxfId="16" priority="17" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L42">
-    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Pending">
+    <cfRule type="containsText" dxfId="15" priority="16" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",L2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1:N1 L2:L42">
-    <cfRule type="containsText" dxfId="2" priority="6" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L43:N1048576">
-    <cfRule type="containsText" dxfId="1" priority="7" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",L43)))</formula>
+  <conditionalFormatting sqref="L47:N1048576">
+    <cfRule type="containsText" dxfId="13" priority="19" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",L47)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="8" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",L43)))</formula>
+    <cfRule type="containsText" dxfId="12" priority="20" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",L47)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L43 H43">
+    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H43)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L43 H43">
+    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H43)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L43 H43">
+    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H43)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L44 H44">
+    <cfRule type="containsText" dxfId="8" priority="7" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H44)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H44)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="9" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H44)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45:H46 L45:L46">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H45)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45:H46">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H45)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45:H46">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H45)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45:H46">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H45)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19474,7 +21014,7 @@
           <x14:formula1>
             <xm:f>Dropdown!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H42 L2:L42</xm:sqref>
+          <xm:sqref>L2:L46 H2:H46</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
added manual testing and counts
</commit_message>
<xml_diff>
--- a/tests/Manual.Integration.Tests.xlsx
+++ b/tests/Manual.Integration.Tests.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Microsoft\ActiveDirectoryTierModel\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5017D7E2-C2B4-4D9B-B4A7-925418F8CE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995A6AE9-9893-4931-ACD9-9D6EFF013CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="555" yWindow="45" windowWidth="37080" windowHeight="20880" xr2:uid="{C99BB6DE-AC80-4F97-BF9F-2DFD37C8A9E7}"/>
+    <workbookView xWindow="25490" yWindow="-3370" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{C99BB6DE-AC80-4F97-BF9F-2DFD37C8A9E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Lab" sheetId="6" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4242" uniqueCount="995">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4302" uniqueCount="1013">
   <si>
     <t>Test Num</t>
   </si>
@@ -3069,6 +3069,60 @@
   </si>
   <si>
     <t>When testing auth silos ensure to remove the 5 URA Deny from the Tier Model Authentication GPOS (Tier 0/1/2 Servers/PAWs) to ensure URA are not denying and only Auth Silos are applying</t>
+  </si>
+  <si>
+    <t>Deploy with Verbose Logging</t>
+  </si>
+  <si>
+    <t>Deploy with Debug Logging</t>
+  </si>
+  <si>
+    <t>Deploy with Verbose and Debug Logging</t>
+  </si>
+  <si>
+    <t>D-42</t>
+  </si>
+  <si>
+    <t>D-43</t>
+  </si>
+  <si>
+    <t>D-44</t>
+  </si>
+  <si>
+    <t>Run deployment script with any other parameters plus -EnableDebug should create the output file</t>
+  </si>
+  <si>
+    <t>Run deployment script with any other parameters plus -EnableVerbose should create the output file</t>
+  </si>
+  <si>
+    <t>Run deployment script with any other parameters plus -EnableVerbose and -EnableDebug should create the output files</t>
+  </si>
+  <si>
+    <t>D-45</t>
+  </si>
+  <si>
+    <t>D-46</t>
+  </si>
+  <si>
+    <t>D-47</t>
+  </si>
+  <si>
+    <t>Audit with Verbose Logging</t>
+  </si>
+  <si>
+    <t>Audit with Debug Logging</t>
+  </si>
+  <si>
+    <t>Audit with Verbose and Debug Logging</t>
+  </si>
+  <si>
+    <t>Run audit script with any other parameters plus -EnableVerbose should create the output file</t>
+  </si>
+  <si>
+    <t>Run audit script with any other parameters plus -EnableDebug should create the output file</t>
+  </si>
+  <si>
+    <t>Run audit script with any other parameters plus -EnableVerbose and -EnableDebug should create the output files</t>
   </si>
 </sst>
 </file>
@@ -3362,7 +3416,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3442,6 +3496,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -3449,7 +3504,7 @@
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="130">
+  <dxfs count="120">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -3462,11 +3517,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3552,16 +3617,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3577,36 +3632,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3662,11 +3687,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3682,31 +3727,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3777,76 +3802,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4359,8 +4314,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BBDC83E0-955E-4441-8E62-48B5AD3B7F7C}" name="Table8" displayName="Table8" ref="A1:O42" totalsRowShown="0" headerRowDxfId="129" headerRowBorderDxfId="128" tableBorderDxfId="127">
-  <autoFilter ref="A1:O42" xr:uid="{BBDC83E0-955E-4441-8E62-48B5AD3B7F7C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BBDC83E0-955E-4441-8E62-48B5AD3B7F7C}" name="Table8" displayName="Table8" ref="A1:O48" totalsRowShown="0" headerRowDxfId="119" headerRowBorderDxfId="118" tableBorderDxfId="117">
+  <autoFilter ref="A1:O48" xr:uid="{BBDC83E0-955E-4441-8E62-48B5AD3B7F7C}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{A4997F13-AC91-46E7-9C27-5D05D8995D60}" name="Test Num"/>
     <tableColumn id="2" xr3:uid="{91F11615-CA80-4054-B5A3-05F0E23A3A98}" name="Role"/>
@@ -4369,13 +4324,13 @@
     <tableColumn id="5" xr3:uid="{1FC76C0A-9A26-4B06-8490-F200EC00E4EF}" name="Member Of"/>
     <tableColumn id="6" xr3:uid="{49812656-8701-4DCA-8B70-59D7F432AD83}" name="Test Device"/>
     <tableColumn id="7" xr3:uid="{2B963348-44AC-44ED-8F30-26C149C9F64D}" name="Steps"/>
-    <tableColumn id="8" xr3:uid="{0D06EF6C-0CD0-4677-876B-3995F790C765}" name="Result 1" dataDxfId="126"/>
-    <tableColumn id="9" xr3:uid="{0B8B0955-473B-49C5-8D3A-A400A4117CBE}" name="Date 1" dataDxfId="125" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{0F470D11-D265-4503-9506-43C538AE2DC1}" name="Tester 1" dataDxfId="124" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{0D06EF6C-0CD0-4677-876B-3995F790C765}" name="Result 1" dataDxfId="116"/>
+    <tableColumn id="9" xr3:uid="{0B8B0955-473B-49C5-8D3A-A400A4117CBE}" name="Date 1" dataDxfId="115" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{0F470D11-D265-4503-9506-43C538AE2DC1}" name="Tester 1" dataDxfId="114" dataCellStyle="Normal"/>
     <tableColumn id="11" xr3:uid="{228CBCFE-86F5-481F-BDEC-40B48BBE889D}" name="Comments 1" dataCellStyle="Normal"/>
-    <tableColumn id="12" xr3:uid="{E5EF96BB-126C-480C-B7FC-77C739DF5B1D}" name="Results 2" dataDxfId="123"/>
+    <tableColumn id="12" xr3:uid="{E5EF96BB-126C-480C-B7FC-77C739DF5B1D}" name="Results 2" dataDxfId="113"/>
     <tableColumn id="13" xr3:uid="{5DB34468-1538-4007-82D6-8EEA8A8C1993}" name="Date 2"/>
-    <tableColumn id="14" xr3:uid="{C18F0626-9D7E-4106-9931-B9986AADE4D0}" name="Tester 2" dataDxfId="122"/>
+    <tableColumn id="14" xr3:uid="{C18F0626-9D7E-4106-9931-B9986AADE4D0}" name="Tester 2" dataDxfId="112"/>
     <tableColumn id="15" xr3:uid="{0B0477E8-6A70-4B4D-B98E-D459B76D22C7}" name="Comments 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4383,96 +4338,96 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FFF45944-2A4D-4033-B755-D7B4507490C2}" name="Table4" displayName="Table4" ref="A1:O87" totalsRowShown="0" headerRowDxfId="121" dataDxfId="120">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FFF45944-2A4D-4033-B755-D7B4507490C2}" name="Table4" displayName="Table4" ref="A1:O87" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
   <autoFilter ref="A1:O87" xr:uid="{FFF45944-2A4D-4033-B755-D7B4507490C2}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{BE52AF1E-BE97-41AD-91ED-DE34C5EE886F}" name="Test Num" dataDxfId="119"/>
-    <tableColumn id="2" xr3:uid="{E7880774-D716-414F-B5F2-C108A070B2D5}" name="Role" dataDxfId="118"/>
-    <tableColumn id="3" xr3:uid="{76377402-3D21-45AB-A9F3-08B60FE18923}" name="Test Case" dataDxfId="117"/>
-    <tableColumn id="4" xr3:uid="{A9117327-F067-4E1B-BBDC-9C9DB8B27F70}" name="Account Tier" dataDxfId="116"/>
-    <tableColumn id="5" xr3:uid="{6FE7F356-C55D-4BD6-B12D-32030CF1EBB0}" name="Member Of" dataDxfId="115"/>
-    <tableColumn id="6" xr3:uid="{A2643D89-0009-48D0-97AD-D861219BCB64}" name="Test Device" dataDxfId="114"/>
-    <tableColumn id="7" xr3:uid="{2DF16A02-3509-4DC9-B46E-952EB6D09826}" name="Steps" dataDxfId="113"/>
-    <tableColumn id="15" xr3:uid="{D3B15A47-8060-4494-9BEC-6113C9237E7B}" name="Result 1" dataDxfId="112"/>
-    <tableColumn id="14" xr3:uid="{D468D462-294C-4B16-A0EC-BE7A78192C80}" name="Date 1" dataDxfId="111"/>
-    <tableColumn id="13" xr3:uid="{DFED3155-8A6F-4EFB-8E41-565AD7D0829E}" name="Tester 1" dataDxfId="110"/>
-    <tableColumn id="12" xr3:uid="{FA56428D-5B55-4936-B617-48C969D29555}" name="Comments 1" dataDxfId="109"/>
-    <tableColumn id="8" xr3:uid="{4AC14231-7F44-4F5A-8DCB-7352EBEF09BF}" name="Results 2" dataDxfId="108"/>
-    <tableColumn id="10" xr3:uid="{A13A5449-5099-47A4-917C-995C610284DC}" name="Date 2" dataDxfId="107"/>
-    <tableColumn id="11" xr3:uid="{2EA75155-8D1B-4327-AAEF-A34C76441CF5}" name="Tester 2" dataDxfId="106"/>
-    <tableColumn id="9" xr3:uid="{781068EC-2F0D-416E-BD14-653C89C646CF}" name="Comments 2" dataDxfId="105"/>
+    <tableColumn id="1" xr3:uid="{BE52AF1E-BE97-41AD-91ED-DE34C5EE886F}" name="Test Num" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{E7880774-D716-414F-B5F2-C108A070B2D5}" name="Role" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{76377402-3D21-45AB-A9F3-08B60FE18923}" name="Test Case" dataDxfId="107"/>
+    <tableColumn id="4" xr3:uid="{A9117327-F067-4E1B-BBDC-9C9DB8B27F70}" name="Account Tier" dataDxfId="106"/>
+    <tableColumn id="5" xr3:uid="{6FE7F356-C55D-4BD6-B12D-32030CF1EBB0}" name="Member Of" dataDxfId="105"/>
+    <tableColumn id="6" xr3:uid="{A2643D89-0009-48D0-97AD-D861219BCB64}" name="Test Device" dataDxfId="104"/>
+    <tableColumn id="7" xr3:uid="{2DF16A02-3509-4DC9-B46E-952EB6D09826}" name="Steps" dataDxfId="103"/>
+    <tableColumn id="15" xr3:uid="{D3B15A47-8060-4494-9BEC-6113C9237E7B}" name="Result 1" dataDxfId="102"/>
+    <tableColumn id="14" xr3:uid="{D468D462-294C-4B16-A0EC-BE7A78192C80}" name="Date 1" dataDxfId="101"/>
+    <tableColumn id="13" xr3:uid="{DFED3155-8A6F-4EFB-8E41-565AD7D0829E}" name="Tester 1" dataDxfId="100"/>
+    <tableColumn id="12" xr3:uid="{FA56428D-5B55-4936-B617-48C969D29555}" name="Comments 1" dataDxfId="99"/>
+    <tableColumn id="8" xr3:uid="{4AC14231-7F44-4F5A-8DCB-7352EBEF09BF}" name="Results 2" dataDxfId="98"/>
+    <tableColumn id="10" xr3:uid="{A13A5449-5099-47A4-917C-995C610284DC}" name="Date 2" dataDxfId="97"/>
+    <tableColumn id="11" xr3:uid="{2EA75155-8D1B-4327-AAEF-A34C76441CF5}" name="Tester 2" dataDxfId="96"/>
+    <tableColumn id="9" xr3:uid="{781068EC-2F0D-416E-BD14-653C89C646CF}" name="Comments 2" dataDxfId="95"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D1C8D22-8799-4789-AC90-A2DA43011B4B}" name="Table3" displayName="Table3" ref="A1:O90" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D1C8D22-8799-4789-AC90-A2DA43011B4B}" name="Table3" displayName="Table3" ref="A1:O90" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93">
   <autoFilter ref="A1:O90" xr:uid="{3D1C8D22-8799-4789-AC90-A2DA43011B4B}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{D09E58BE-FEF9-41DE-9D8D-1DADA7CB1A3E}" name="Test Num" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{7918EE24-0094-48F6-8ED5-8FB237D184F0}" name="Role" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{C7183E2C-E9B9-42AC-A164-5F1998E926CC}" name="Test Case" dataDxfId="100"/>
-    <tableColumn id="4" xr3:uid="{9C400D12-E338-4EFE-A7C1-92B5F198A30B}" name="Account Tier" dataDxfId="99"/>
-    <tableColumn id="5" xr3:uid="{9FB3EAFA-D413-4020-9923-30FBEA1C2483}" name="Member Of" dataDxfId="98"/>
-    <tableColumn id="6" xr3:uid="{1F963AD9-DBB5-44C8-BAC6-ADB071A246EC}" name="Test Device" dataDxfId="97"/>
-    <tableColumn id="7" xr3:uid="{961A93C3-EF44-4D30-BA51-3AB1F368149E}" name="Steps" dataDxfId="96"/>
-    <tableColumn id="15" xr3:uid="{64EBB73C-E234-4AEA-BF57-BA56C45781A4}" name="Result 1" dataDxfId="95"/>
-    <tableColumn id="14" xr3:uid="{57728B78-D8B9-469F-BE14-1F7300E25B0A}" name="Date 1" dataDxfId="94"/>
-    <tableColumn id="13" xr3:uid="{A85C0F5E-3B6E-49C0-B6F0-70D0979863B9}" name="Tester 1" dataDxfId="93"/>
-    <tableColumn id="12" xr3:uid="{4B38473F-A7B1-469C-A50C-01068E9ED7CE}" name="Comments 1" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{4F269C65-5B7E-456A-A494-D44AB144D363}" name="Results 2" dataDxfId="91"/>
-    <tableColumn id="10" xr3:uid="{2109691A-4EDC-458B-A336-6B6E190B9A92}" name="Date 2" dataDxfId="90"/>
-    <tableColumn id="11" xr3:uid="{930C7486-8059-4A94-8E80-E4541438DEB4}" name="Tester 2" dataDxfId="89"/>
-    <tableColumn id="9" xr3:uid="{4B6480AC-F6F9-44B9-8DA4-A907BB1A0276}" name="Comments 2" dataDxfId="88"/>
+    <tableColumn id="1" xr3:uid="{D09E58BE-FEF9-41DE-9D8D-1DADA7CB1A3E}" name="Test Num" dataDxfId="92"/>
+    <tableColumn id="2" xr3:uid="{7918EE24-0094-48F6-8ED5-8FB237D184F0}" name="Role" dataDxfId="91"/>
+    <tableColumn id="3" xr3:uid="{C7183E2C-E9B9-42AC-A164-5F1998E926CC}" name="Test Case" dataDxfId="90"/>
+    <tableColumn id="4" xr3:uid="{9C400D12-E338-4EFE-A7C1-92B5F198A30B}" name="Account Tier" dataDxfId="89"/>
+    <tableColumn id="5" xr3:uid="{9FB3EAFA-D413-4020-9923-30FBEA1C2483}" name="Member Of" dataDxfId="88"/>
+    <tableColumn id="6" xr3:uid="{1F963AD9-DBB5-44C8-BAC6-ADB071A246EC}" name="Test Device" dataDxfId="87"/>
+    <tableColumn id="7" xr3:uid="{961A93C3-EF44-4D30-BA51-3AB1F368149E}" name="Steps" dataDxfId="86"/>
+    <tableColumn id="15" xr3:uid="{64EBB73C-E234-4AEA-BF57-BA56C45781A4}" name="Result 1" dataDxfId="85"/>
+    <tableColumn id="14" xr3:uid="{57728B78-D8B9-469F-BE14-1F7300E25B0A}" name="Date 1" dataDxfId="84"/>
+    <tableColumn id="13" xr3:uid="{A85C0F5E-3B6E-49C0-B6F0-70D0979863B9}" name="Tester 1" dataDxfId="83"/>
+    <tableColumn id="12" xr3:uid="{4B38473F-A7B1-469C-A50C-01068E9ED7CE}" name="Comments 1" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{4F269C65-5B7E-456A-A494-D44AB144D363}" name="Results 2" dataDxfId="81"/>
+    <tableColumn id="10" xr3:uid="{2109691A-4EDC-458B-A336-6B6E190B9A92}" name="Date 2" dataDxfId="80"/>
+    <tableColumn id="11" xr3:uid="{930C7486-8059-4A94-8E80-E4541438DEB4}" name="Tester 2" dataDxfId="79"/>
+    <tableColumn id="9" xr3:uid="{4B6480AC-F6F9-44B9-8DA4-A907BB1A0276}" name="Comments 2" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6CB453EC-9F38-4A1A-841E-12373A0046E8}" name="Table2" displayName="Table2" ref="A1:O118" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6CB453EC-9F38-4A1A-841E-12373A0046E8}" name="Table2" displayName="Table2" ref="A1:O118" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:O118" xr:uid="{6CB453EC-9F38-4A1A-841E-12373A0046E8}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{6F968ADA-C366-45BB-8076-11A6E132598D}" name="Test Num" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{1CF9D31D-A3E8-43CB-9C53-1B5CA334451D}" name="Role" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{A4586D46-3561-4DB2-A5CD-82F11E112E36}" name="Test Case" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{3074E7FF-6671-4AF2-98D7-4B64EA286C21}" name="Account Tier" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{61DC852D-ACBB-4250-AE54-F784DBA0124F}" name="Member Of" dataDxfId="81"/>
-    <tableColumn id="6" xr3:uid="{A4A28542-1156-415C-B9A6-26B2C64571C8}" name="Test Device" dataDxfId="80"/>
-    <tableColumn id="7" xr3:uid="{508667C8-E7DC-4B36-B730-1BF07B072B26}" name="Steps" dataDxfId="79"/>
-    <tableColumn id="15" xr3:uid="{98B63D13-4B1B-4929-A507-3B339C9178DC}" name="Result 1" dataDxfId="78"/>
-    <tableColumn id="14" xr3:uid="{0960049F-6624-4EF2-A9BE-6C4BF1BF0B30}" name="Date 1" dataDxfId="77"/>
-    <tableColumn id="13" xr3:uid="{B8038056-A835-4C98-83D2-9F7F811DA5B5}" name="Tester 1" dataDxfId="76"/>
-    <tableColumn id="12" xr3:uid="{7A4FCB71-BD95-4A2A-9499-EE33978E1B72}" name="Comment 1" dataDxfId="75"/>
-    <tableColumn id="8" xr3:uid="{962A06FB-258E-4DB6-B7AD-C09A30D77672}" name="Results 2" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{385794D4-4829-4203-BE5E-17ECE94BC5D3}" name="Date 2" dataDxfId="73"/>
-    <tableColumn id="11" xr3:uid="{F0A1DEEA-8A69-45E5-9D9F-58AF6D63896D}" name="Tester 2" dataDxfId="72"/>
-    <tableColumn id="9" xr3:uid="{255C1446-C13E-4C8B-B25C-201918325FA2}" name="Comments 2" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{6F968ADA-C366-45BB-8076-11A6E132598D}" name="Test Num" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{1CF9D31D-A3E8-43CB-9C53-1B5CA334451D}" name="Role" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{A4586D46-3561-4DB2-A5CD-82F11E112E36}" name="Test Case" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{3074E7FF-6671-4AF2-98D7-4B64EA286C21}" name="Account Tier" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{61DC852D-ACBB-4250-AE54-F784DBA0124F}" name="Member Of" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{A4A28542-1156-415C-B9A6-26B2C64571C8}" name="Test Device" dataDxfId="70"/>
+    <tableColumn id="7" xr3:uid="{508667C8-E7DC-4B36-B730-1BF07B072B26}" name="Steps" dataDxfId="69"/>
+    <tableColumn id="15" xr3:uid="{98B63D13-4B1B-4929-A507-3B339C9178DC}" name="Result 1" dataDxfId="68"/>
+    <tableColumn id="14" xr3:uid="{0960049F-6624-4EF2-A9BE-6C4BF1BF0B30}" name="Date 1" dataDxfId="67"/>
+    <tableColumn id="13" xr3:uid="{B8038056-A835-4C98-83D2-9F7F811DA5B5}" name="Tester 1" dataDxfId="66"/>
+    <tableColumn id="12" xr3:uid="{7A4FCB71-BD95-4A2A-9499-EE33978E1B72}" name="Comment 1" dataDxfId="65"/>
+    <tableColumn id="8" xr3:uid="{962A06FB-258E-4DB6-B7AD-C09A30D77672}" name="Results 2" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{385794D4-4829-4203-BE5E-17ECE94BC5D3}" name="Date 2" dataDxfId="63"/>
+    <tableColumn id="11" xr3:uid="{F0A1DEEA-8A69-45E5-9D9F-58AF6D63896D}" name="Tester 2" dataDxfId="62"/>
+    <tableColumn id="9" xr3:uid="{255C1446-C13E-4C8B-B25C-201918325FA2}" name="Comments 2" dataDxfId="61"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EB17A5CC-E408-4C9A-B5B1-6D8E779BD4FF}" name="Table1" displayName="Table1" ref="A1:O46" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EB17A5CC-E408-4C9A-B5B1-6D8E779BD4FF}" name="Table1" displayName="Table1" ref="A1:O46" totalsRowShown="0" headerRowDxfId="60" dataDxfId="59">
   <autoFilter ref="A1:O46" xr:uid="{EB17A5CC-E408-4C9A-B5B1-6D8E779BD4FF}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{823BC357-BB93-4F33-BD5C-CA74E34526D5}" name="Test Num" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{17424961-31D2-4C05-8CB9-9657B47F8534}" name="Role" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{AF7EE82B-D8B0-461F-AC7A-26F79D6F1400}" name="Test Case" dataDxfId="66"/>
-    <tableColumn id="4" xr3:uid="{7C7C56AD-F058-48C0-B4E4-CCCAFF2251BB}" name="Account Tier" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{DED0F04D-B39D-4D1D-827C-FA435FA02FB5}" name="Member Of" dataDxfId="64"/>
-    <tableColumn id="6" xr3:uid="{89BD421D-B187-43BD-97FE-5DC073DE828B}" name="Test Device" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{A56500EF-650E-4E5B-8835-999502D63C09}" name="Steps" dataDxfId="62"/>
-    <tableColumn id="15" xr3:uid="{9EAAD511-E661-49CF-A644-79E3D2286F82}" name="Result 1" dataDxfId="61"/>
-    <tableColumn id="14" xr3:uid="{D147186E-F9DE-4DEE-AC48-717CF1F2EFFF}" name="Date 1" dataDxfId="60"/>
-    <tableColumn id="13" xr3:uid="{005F10CF-A98F-4680-A807-A3DA2AC11987}" name="Tester 1" dataDxfId="59"/>
-    <tableColumn id="12" xr3:uid="{B10B013E-B707-45F1-A349-E3949E0318B6}" name="Comments 1" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{B0760FD3-784D-4B94-9349-CCBCF60DDBDF}" name="Results 2" dataDxfId="57"/>
-    <tableColumn id="10" xr3:uid="{CF7BC678-11B8-4277-8A7D-BE27B1DD3883}" name="Date 2" dataDxfId="56"/>
-    <tableColumn id="11" xr3:uid="{E153E44B-CE3E-468C-BD29-0EC84853E492}" name="Tester 2" dataDxfId="55"/>
-    <tableColumn id="9" xr3:uid="{56D1854D-5874-4A46-8106-061E8E3D40DF}" name="Comments 2" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{823BC357-BB93-4F33-BD5C-CA74E34526D5}" name="Test Num" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{17424961-31D2-4C05-8CB9-9657B47F8534}" name="Role" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{AF7EE82B-D8B0-461F-AC7A-26F79D6F1400}" name="Test Case" dataDxfId="56"/>
+    <tableColumn id="4" xr3:uid="{7C7C56AD-F058-48C0-B4E4-CCCAFF2251BB}" name="Account Tier" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{DED0F04D-B39D-4D1D-827C-FA435FA02FB5}" name="Member Of" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{89BD421D-B187-43BD-97FE-5DC073DE828B}" name="Test Device" dataDxfId="53"/>
+    <tableColumn id="7" xr3:uid="{A56500EF-650E-4E5B-8835-999502D63C09}" name="Steps" dataDxfId="52"/>
+    <tableColumn id="15" xr3:uid="{9EAAD511-E661-49CF-A644-79E3D2286F82}" name="Result 1" dataDxfId="51"/>
+    <tableColumn id="14" xr3:uid="{D147186E-F9DE-4DEE-AC48-717CF1F2EFFF}" name="Date 1" dataDxfId="50"/>
+    <tableColumn id="13" xr3:uid="{005F10CF-A98F-4680-A807-A3DA2AC11987}" name="Tester 1" dataDxfId="49"/>
+    <tableColumn id="12" xr3:uid="{B10B013E-B707-45F1-A349-E3949E0318B6}" name="Comments 1" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{B0760FD3-784D-4B94-9349-CCBCF60DDBDF}" name="Results 2" dataDxfId="47"/>
+    <tableColumn id="10" xr3:uid="{CF7BC678-11B8-4277-8A7D-BE27B1DD3883}" name="Date 2" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{E153E44B-CE3E-468C-BD29-0EC84853E492}" name="Tester 2" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{56D1854D-5874-4A46-8106-061E8E3D40DF}" name="Comments 2" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4867,11 +4822,11 @@
       </c>
       <c r="J2" s="10">
         <f>COUNTIF(Deploy!L:L,"Pending")+COUNTIF('Tier 0'!L:L,"Pending")+COUNTIF('Tier 1'!L:L,"Pending")+COUNTIF('Tier 2'!L:L,"Pending")+COUNTIF('Outside TM'!L:L,"Pending")</f>
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="K2" s="15">
         <f>SUM(I2:J2)</f>
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -4933,7 +4888,7 @@
       </c>
       <c r="I4" s="18">
         <f>COUNTIF(Deploy!H:H,"Pass")+COUNTIF('Tier 0'!H:H,"Pass")+COUNTIF('Tier 1'!H:H,"Pass")+COUNTIF('Tier 2'!H:H,"Pass")+COUNTIF('Outside TM'!H:H,"Pass")</f>
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="J4" s="18">
         <f>COUNTIF(Deploy!L:L,"Pass")+COUNTIF('Tier 0'!L:L,"Pass")+COUNTIF('Tier 1'!L:L,"Pass")+COUNTIF('Tier 2'!L:L,"Pass")+COUNTIF('Outside TM'!L:L,"Pass")</f>
@@ -4941,7 +4896,7 @@
       </c>
       <c r="K4" s="19">
         <f t="shared" si="0"/>
-        <v>604</v>
+        <v>610</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -5244,17 +5199,17 @@
     <mergeCell ref="A28:D28"/>
   </mergeCells>
   <conditionalFormatting sqref="I2:K2">
-    <cfRule type="cellIs" dxfId="53" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="43" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3:K3">
-    <cfRule type="cellIs" dxfId="52" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4:K4">
-    <cfRule type="cellIs" dxfId="51" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
       <formula>132</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5271,7 +5226,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D89F1577-A29D-498F-A7FA-5988ED9F0B5A}">
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -6236,10 +6191,10 @@
         <v>876</v>
       </c>
       <c r="B25" t="s">
-        <v>716</v>
+        <v>663</v>
       </c>
       <c r="C25" t="s">
-        <v>654</v>
+        <v>995</v>
       </c>
       <c r="D25" t="s">
         <v>88</v>
@@ -6251,36 +6206,32 @@
         <v>306</v>
       </c>
       <c r="G25" t="s">
-        <v>685</v>
+        <v>1002</v>
       </c>
       <c r="H25" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I25" s="8">
-        <v>46072</v>
+        <v>46273</v>
       </c>
       <c r="J25" s="7" t="s">
         <v>704</v>
       </c>
+      <c r="K25" s="29"/>
       <c r="L25" s="20" t="s">
-        <v>372</v>
-      </c>
-      <c r="M25" s="8">
-        <v>46120</v>
-      </c>
-      <c r="N25" s="7" t="s">
-        <v>705</v>
-      </c>
+        <v>594</v>
+      </c>
+      <c r="M25" s="8"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>877</v>
       </c>
       <c r="B26" t="s">
-        <v>716</v>
+        <v>663</v>
       </c>
       <c r="C26" t="s">
-        <v>717</v>
+        <v>996</v>
       </c>
       <c r="D26" t="s">
         <v>88</v>
@@ -6292,17 +6243,18 @@
         <v>306</v>
       </c>
       <c r="G26" t="s">
-        <v>718</v>
+        <v>1001</v>
       </c>
       <c r="H26" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I26" s="8">
-        <v>46177</v>
+        <v>46273</v>
       </c>
       <c r="J26" s="7" t="s">
         <v>704</v>
       </c>
+      <c r="K26" s="29"/>
       <c r="L26" s="20" t="s">
         <v>594</v>
       </c>
@@ -6313,10 +6265,10 @@
         <v>878</v>
       </c>
       <c r="B27" t="s">
-        <v>716</v>
+        <v>663</v>
       </c>
       <c r="C27" t="s">
-        <v>781</v>
+        <v>997</v>
       </c>
       <c r="D27" t="s">
         <v>88</v>
@@ -6328,17 +6280,18 @@
         <v>306</v>
       </c>
       <c r="G27" t="s">
-        <v>783</v>
+        <v>1003</v>
       </c>
       <c r="H27" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I27" s="8">
-        <v>46218</v>
+        <v>46273</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>704</v>
       </c>
+      <c r="K27" s="29"/>
       <c r="L27" s="20" t="s">
         <v>594</v>
       </c>
@@ -6352,7 +6305,7 @@
         <v>716</v>
       </c>
       <c r="C28" t="s">
-        <v>828</v>
+        <v>654</v>
       </c>
       <c r="D28" t="s">
         <v>88</v>
@@ -6364,21 +6317,26 @@
         <v>306</v>
       </c>
       <c r="G28" t="s">
-        <v>829</v>
+        <v>685</v>
       </c>
       <c r="H28" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I28" s="8">
-        <v>46249</v>
+        <v>46072</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>704</v>
       </c>
       <c r="L28" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="M28" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="M28" s="8">
+        <v>46120</v>
+      </c>
+      <c r="N28" s="7" t="s">
+        <v>705</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -6388,7 +6346,7 @@
         <v>716</v>
       </c>
       <c r="C29" t="s">
-        <v>851</v>
+        <v>717</v>
       </c>
       <c r="D29" t="s">
         <v>88</v>
@@ -6400,13 +6358,13 @@
         <v>306</v>
       </c>
       <c r="G29" t="s">
-        <v>850</v>
+        <v>718</v>
       </c>
       <c r="H29" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I29" s="8">
-        <v>46261</v>
+        <v>46177</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>704</v>
@@ -6424,7 +6382,7 @@
         <v>716</v>
       </c>
       <c r="C30" t="s">
-        <v>655</v>
+        <v>781</v>
       </c>
       <c r="D30" t="s">
         <v>88</v>
@@ -6436,26 +6394,21 @@
         <v>306</v>
       </c>
       <c r="G30" t="s">
-        <v>686</v>
+        <v>783</v>
       </c>
       <c r="H30" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I30" s="8">
-        <v>46072</v>
+        <v>46218</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>704</v>
       </c>
       <c r="L30" s="20" t="s">
-        <v>372</v>
-      </c>
-      <c r="M30" s="8">
-        <v>46120</v>
-      </c>
-      <c r="N30" s="7" t="s">
-        <v>705</v>
-      </c>
+        <v>594</v>
+      </c>
+      <c r="M30" s="8"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
@@ -6465,7 +6418,7 @@
         <v>716</v>
       </c>
       <c r="C31" t="s">
-        <v>656</v>
+        <v>828</v>
       </c>
       <c r="D31" t="s">
         <v>88</v>
@@ -6477,26 +6430,21 @@
         <v>306</v>
       </c>
       <c r="G31" t="s">
-        <v>687</v>
+        <v>829</v>
       </c>
       <c r="H31" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I31" s="8">
-        <v>46072</v>
+        <v>46249</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>704</v>
       </c>
       <c r="L31" s="20" t="s">
-        <v>372</v>
-      </c>
-      <c r="M31" s="8">
-        <v>46120</v>
-      </c>
-      <c r="N31" s="7" t="s">
-        <v>705</v>
-      </c>
+        <v>594</v>
+      </c>
+      <c r="M31" s="8"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -6506,7 +6454,7 @@
         <v>716</v>
       </c>
       <c r="C32" t="s">
-        <v>657</v>
+        <v>851</v>
       </c>
       <c r="D32" t="s">
         <v>88</v>
@@ -6518,26 +6466,21 @@
         <v>306</v>
       </c>
       <c r="G32" t="s">
-        <v>688</v>
+        <v>850</v>
       </c>
       <c r="H32" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I32" s="8">
-        <v>46072</v>
+        <v>46261</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>704</v>
       </c>
       <c r="L32" s="20" t="s">
-        <v>372</v>
-      </c>
-      <c r="M32" s="8">
-        <v>46120</v>
-      </c>
-      <c r="N32" s="7" t="s">
-        <v>705</v>
-      </c>
+        <v>594</v>
+      </c>
+      <c r="M32" s="8"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
@@ -6547,7 +6490,7 @@
         <v>716</v>
       </c>
       <c r="C33" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="D33" t="s">
         <v>88</v>
@@ -6559,7 +6502,7 @@
         <v>306</v>
       </c>
       <c r="G33" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="H33" s="20" t="s">
         <v>372</v>
@@ -6588,7 +6531,7 @@
         <v>716</v>
       </c>
       <c r="C34" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="D34" t="s">
         <v>88</v>
@@ -6600,7 +6543,7 @@
         <v>306</v>
       </c>
       <c r="G34" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="H34" s="20" t="s">
         <v>372</v>
@@ -6629,7 +6572,7 @@
         <v>716</v>
       </c>
       <c r="C35" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="D35" t="s">
         <v>88</v>
@@ -6641,7 +6584,7 @@
         <v>306</v>
       </c>
       <c r="G35" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="H35" s="20" t="s">
         <v>372</v>
@@ -6670,7 +6613,7 @@
         <v>716</v>
       </c>
       <c r="C36" t="s">
-        <v>719</v>
+        <v>658</v>
       </c>
       <c r="D36" t="s">
         <v>88</v>
@@ -6682,21 +6625,26 @@
         <v>306</v>
       </c>
       <c r="G36" t="s">
-        <v>722</v>
+        <v>692</v>
       </c>
       <c r="H36" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I36" s="8">
-        <v>46177</v>
+        <v>46072</v>
       </c>
       <c r="J36" s="7" t="s">
         <v>704</v>
       </c>
       <c r="L36" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="M36" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="M36" s="8">
+        <v>46120</v>
+      </c>
+      <c r="N36" s="7" t="s">
+        <v>705</v>
+      </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
@@ -6706,7 +6654,7 @@
         <v>716</v>
       </c>
       <c r="C37" t="s">
-        <v>720</v>
+        <v>659</v>
       </c>
       <c r="D37" t="s">
         <v>88</v>
@@ -6718,21 +6666,26 @@
         <v>306</v>
       </c>
       <c r="G37" t="s">
-        <v>723</v>
+        <v>689</v>
       </c>
       <c r="H37" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I37" s="8">
-        <v>46177</v>
+        <v>46072</v>
       </c>
       <c r="J37" s="7" t="s">
         <v>704</v>
       </c>
       <c r="L37" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="M37" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="M37" s="8">
+        <v>46120</v>
+      </c>
+      <c r="N37" s="7" t="s">
+        <v>705</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
@@ -6742,7 +6695,7 @@
         <v>716</v>
       </c>
       <c r="C38" t="s">
-        <v>721</v>
+        <v>660</v>
       </c>
       <c r="D38" t="s">
         <v>88</v>
@@ -6754,21 +6707,26 @@
         <v>306</v>
       </c>
       <c r="G38" t="s">
-        <v>724</v>
+        <v>690</v>
       </c>
       <c r="H38" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I38" s="8">
-        <v>46177</v>
+        <v>46072</v>
       </c>
       <c r="J38" s="7" t="s">
         <v>704</v>
       </c>
       <c r="L38" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="M38" s="8"/>
+        <v>372</v>
+      </c>
+      <c r="M38" s="8">
+        <v>46120</v>
+      </c>
+      <c r="N38" s="7" t="s">
+        <v>705</v>
+      </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
@@ -6778,7 +6736,7 @@
         <v>716</v>
       </c>
       <c r="C39" t="s">
-        <v>784</v>
+        <v>719</v>
       </c>
       <c r="D39" t="s">
         <v>88</v>
@@ -6790,13 +6748,13 @@
         <v>306</v>
       </c>
       <c r="G39" t="s">
-        <v>785</v>
+        <v>722</v>
       </c>
       <c r="H39" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I39" s="8">
-        <v>46218</v>
+        <v>46177</v>
       </c>
       <c r="J39" s="7" t="s">
         <v>704</v>
@@ -6814,7 +6772,7 @@
         <v>716</v>
       </c>
       <c r="C40" t="s">
-        <v>847</v>
+        <v>720</v>
       </c>
       <c r="D40" t="s">
         <v>88</v>
@@ -6826,13 +6784,13 @@
         <v>306</v>
       </c>
       <c r="G40" t="s">
-        <v>830</v>
+        <v>723</v>
       </c>
       <c r="H40" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I40" s="8">
-        <v>46249</v>
+        <v>46177</v>
       </c>
       <c r="J40" s="7" t="s">
         <v>704</v>
@@ -6850,7 +6808,7 @@
         <v>716</v>
       </c>
       <c r="C41" t="s">
-        <v>848</v>
+        <v>721</v>
       </c>
       <c r="D41" t="s">
         <v>88</v>
@@ -6862,13 +6820,13 @@
         <v>306</v>
       </c>
       <c r="G41" t="s">
-        <v>849</v>
+        <v>724</v>
       </c>
       <c r="H41" s="20" t="s">
         <v>372</v>
       </c>
       <c r="I41" s="8">
-        <v>46261</v>
+        <v>46177</v>
       </c>
       <c r="J41" s="7" t="s">
         <v>704</v>
@@ -6886,7 +6844,7 @@
         <v>716</v>
       </c>
       <c r="C42" t="s">
-        <v>661</v>
+        <v>784</v>
       </c>
       <c r="D42" t="s">
         <v>88</v>
@@ -6898,45 +6856,264 @@
         <v>306</v>
       </c>
       <c r="G42" t="s">
+        <v>785</v>
+      </c>
+      <c r="H42" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I42" s="8">
+        <v>46218</v>
+      </c>
+      <c r="J42" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="L42" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="M42" s="8"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>998</v>
+      </c>
+      <c r="B43" t="s">
+        <v>716</v>
+      </c>
+      <c r="C43" t="s">
+        <v>847</v>
+      </c>
+      <c r="D43" t="s">
+        <v>88</v>
+      </c>
+      <c r="E43" t="s">
+        <v>482</v>
+      </c>
+      <c r="F43" t="s">
+        <v>306</v>
+      </c>
+      <c r="G43" t="s">
+        <v>830</v>
+      </c>
+      <c r="H43" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I43" s="8">
+        <v>46249</v>
+      </c>
+      <c r="J43" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="L43" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="M43" s="8"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>999</v>
+      </c>
+      <c r="B44" t="s">
+        <v>716</v>
+      </c>
+      <c r="C44" t="s">
+        <v>848</v>
+      </c>
+      <c r="D44" t="s">
+        <v>88</v>
+      </c>
+      <c r="E44" t="s">
+        <v>482</v>
+      </c>
+      <c r="F44" t="s">
+        <v>306</v>
+      </c>
+      <c r="G44" t="s">
+        <v>849</v>
+      </c>
+      <c r="H44" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I44" s="8">
+        <v>46261</v>
+      </c>
+      <c r="J44" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="L44" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="M44" s="8"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B45" t="s">
+        <v>716</v>
+      </c>
+      <c r="C45" t="s">
+        <v>661</v>
+      </c>
+      <c r="D45" t="s">
+        <v>88</v>
+      </c>
+      <c r="E45" t="s">
+        <v>482</v>
+      </c>
+      <c r="F45" t="s">
+        <v>306</v>
+      </c>
+      <c r="G45" t="s">
         <v>691</v>
       </c>
-      <c r="H42" s="20" t="s">
-        <v>372</v>
-      </c>
-      <c r="I42" s="8">
-        <v>46072</v>
-      </c>
-      <c r="J42" s="7" t="s">
-        <v>704</v>
-      </c>
-      <c r="L42" s="20" t="s">
-        <v>372</v>
-      </c>
-      <c r="M42" s="8">
-        <v>46120</v>
-      </c>
-      <c r="N42" s="7" t="s">
-        <v>705</v>
-      </c>
+      <c r="H45" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I45" s="8">
+        <v>46072</v>
+      </c>
+      <c r="J45" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="L45" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="M45" s="8">
+        <v>46120</v>
+      </c>
+      <c r="N45" s="7" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B46" t="s">
+        <v>716</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D46" t="s">
+        <v>89</v>
+      </c>
+      <c r="E46" t="s">
+        <v>482</v>
+      </c>
+      <c r="F46" t="s">
+        <v>306</v>
+      </c>
+      <c r="G46" t="s">
+        <v>1010</v>
+      </c>
+      <c r="H46" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I46" s="8">
+        <v>46273</v>
+      </c>
+      <c r="J46" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="K46" s="29"/>
+      <c r="L46" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="M46" s="8"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B47" t="s">
+        <v>716</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1008</v>
+      </c>
+      <c r="D47" t="s">
+        <v>3</v>
+      </c>
+      <c r="E47" t="s">
+        <v>482</v>
+      </c>
+      <c r="F47" t="s">
+        <v>306</v>
+      </c>
+      <c r="G47" t="s">
+        <v>1011</v>
+      </c>
+      <c r="H47" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I47" s="8">
+        <v>46273</v>
+      </c>
+      <c r="J47" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="K47" s="29"/>
+      <c r="L47" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="M47" s="8"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B48" t="s">
+        <v>716</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D48" t="s">
+        <v>749</v>
+      </c>
+      <c r="E48" t="s">
+        <v>482</v>
+      </c>
+      <c r="F48" t="s">
+        <v>306</v>
+      </c>
+      <c r="G48" t="s">
+        <v>1012</v>
+      </c>
+      <c r="H48" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="I48" s="8">
+        <v>46273</v>
+      </c>
+      <c r="J48" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="K48" s="29"/>
+      <c r="L48" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="M48" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="L2:L42 H2:H42">
-    <cfRule type="containsText" dxfId="50" priority="4" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="H2:H48 L2:L48">
+    <cfRule type="containsText" dxfId="40" priority="4" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="49" priority="5" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="39" priority="5" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="48" priority="6" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="38" priority="6" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1:N1">
-    <cfRule type="containsText" dxfId="47" priority="7" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="37" priority="7" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="8" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="36" priority="8" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6951,7 +7128,7 @@
           <x14:formula1>
             <xm:f>Dropdown!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L42 H2:H42</xm:sqref>
+          <xm:sqref>H2:H48 L2:L48</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -10535,18 +10712,18 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="L1:N1 L88:N1048576 L2:L87 H2:H87">
-    <cfRule type="containsText" dxfId="45" priority="7" operator="containsText" text="Fail">
+  <conditionalFormatting sqref="H2:H87 L2:L87 L1:N1 L88:N1048576">
+    <cfRule type="containsText" dxfId="35" priority="7" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L87 H2:H87">
-    <cfRule type="containsText" dxfId="44" priority="4" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="H2:H87 L2:L87">
+    <cfRule type="containsText" dxfId="34" priority="4" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1:N1 L88:N1048576 L2:L87 H2:H87">
-    <cfRule type="containsText" dxfId="43" priority="8" operator="containsText" text="Pass">
+  <conditionalFormatting sqref="L1:N1 H2:H87 L2:L87 L88:N1048576">
+    <cfRule type="containsText" dxfId="33" priority="8" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14168,46 +14345,42 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H87 H89:H90 L2:L90">
-    <cfRule type="containsText" dxfId="42" priority="4" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="H2:H90">
+    <cfRule type="containsText" dxfId="32" priority="1" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="41" priority="5" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="31" priority="2" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="6" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L90">
+    <cfRule type="containsText" dxfId="29" priority="4" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",L2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",L2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="27" priority="6" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",L2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L1:N1">
-    <cfRule type="containsText" dxfId="39" priority="11" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="26" priority="11" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="12" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="25" priority="12" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L91:N1048576">
-    <cfRule type="containsText" dxfId="37" priority="13" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="24" priority="13" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L91)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="36" priority="14" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="23" priority="14" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L91)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
-    <cfRule type="containsText" dxfId="35" priority="2" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H88)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
-    <cfRule type="containsText" dxfId="34" priority="1" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H88)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
-    <cfRule type="containsText" dxfId="33" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H88)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19023,61 +19196,53 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="L2:L118 H2:H118">
-    <cfRule type="containsText" dxfId="32" priority="7" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="H2:H118 L2:L118">
+    <cfRule type="containsText" dxfId="22" priority="7" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="21" priority="8" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="9" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H105">
+    <cfRule type="containsText" dxfId="19" priority="4" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H105)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="5" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H105)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H105)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H107:H118">
+    <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H107)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H107)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H107)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L1:N1">
-    <cfRule type="containsText" dxfId="29" priority="23" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="13" priority="23" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="24" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="12" priority="24" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L119:N1048576">
-    <cfRule type="containsText" dxfId="27" priority="35" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="11" priority="35" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L119)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="36" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="10" priority="36" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L119)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H105 H107:H116">
-    <cfRule type="containsText" dxfId="25" priority="5" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H105)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H105 H107:H116">
-    <cfRule type="containsText" dxfId="24" priority="4" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H105)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H105 H107:H116">
-    <cfRule type="containsText" dxfId="23" priority="6" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H105)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H117:H118">
-    <cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H117)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H117:H118">
-    <cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H117)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H117:H118">
-    <cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H117)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20775,7 +20940,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>989</v>
       </c>
@@ -20810,7 +20975,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>990</v>
       </c>
@@ -20917,90 +21082,42 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H2:H42">
-    <cfRule type="containsText" dxfId="19" priority="13" operator="containsText" text="Pending">
+  <conditionalFormatting sqref="H2:H46 L2:L46">
+    <cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="14" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="15" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="7" priority="6" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1:N1 L2:L42">
-    <cfRule type="containsText" dxfId="16" priority="17" operator="containsText" text="Fail">
+  <conditionalFormatting sqref="H45:H46">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",H45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",H45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",H45)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L1:N1">
+    <cfRule type="containsText" dxfId="3" priority="17" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L1)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L42">
-    <cfRule type="containsText" dxfId="15" priority="16" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",L2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L1:N1 L2:L42">
-    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="2" priority="18" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L47:N1048576">
-    <cfRule type="containsText" dxfId="13" priority="19" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="1" priority="19" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",L47)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="20" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="0" priority="20" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",L47)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L43 H43">
-    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H43)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L43 H43">
-    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H43)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L43 H43">
-    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H43)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L44 H44">
-    <cfRule type="containsText" dxfId="8" priority="7" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H44)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H44)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="9" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H44)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H45:H46 L45:L46">
-    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H45)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H45)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H45)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H45:H46">
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",H45)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H45:H46">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",H45)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H45:H46">
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",H45)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>